<commit_message>
Auto update AlphaForge data
</commit_message>
<xml_diff>
--- a/AlphaForge_Action_Plan.xlsx
+++ b/AlphaForge_Action_Plan.xlsx
@@ -776,10 +776,10 @@
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>61</v>
+        <v>61.1</v>
       </c>
       <c r="F2" t="n">
-        <v>65</v>
+        <v>65.2</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>score 61.0; priority 65.0; trend: Constructive; entry zone: Constructive entry zone; risk flag: Medium-high risk</t>
+          <t>score 61.1; priority 65.2; trend: Constructive; entry zone: Constructive entry zone; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -808,12 +808,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>RBOT.MI: scenario base Hold / Monitor, score 61.0, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -1.6%.</t>
+          <t>RBOT.MI: scenario base Hold / Monitor, score 61.1, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -1.4%.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -864,10 +864,10 @@
         </is>
       </c>
       <c r="Y2" t="n">
-        <v>-3.17</v>
+        <v>-2.97</v>
       </c>
       <c r="Z2" t="n">
-        <v>34.71</v>
+        <v>34.98</v>
       </c>
       <c r="AA2" t="n">
         <v>22.52</v>
@@ -888,65 +888,65 @@
         </is>
       </c>
       <c r="AG2" t="n">
-        <v>17.838</v>
+        <v>17.874</v>
       </c>
       <c r="AH2" t="n">
         <v>50.8</v>
       </c>
       <c r="AI2" t="n">
-        <v>72</v>
+        <v>72.5</v>
       </c>
       <c r="AJ2" t="n">
         <v>44.5</v>
       </c>
       <c r="AK2" t="n">
-        <v>77.40000000000001</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="AL2" t="n">
-        <v>-6.2</v>
+        <v>-6.02</v>
       </c>
       <c r="AM2" t="n">
-        <v>29.52</v>
+        <v>29.79</v>
       </c>
       <c r="AN2" t="n">
-        <v>18.85</v>
+        <v>18.93</v>
       </c>
       <c r="AO2" t="n">
         <v>0.84</v>
       </c>
       <c r="AP2" t="n">
-        <v>18.1279</v>
+        <v>18.1286</v>
       </c>
       <c r="AQ2" t="n">
-        <v>16.0374</v>
+        <v>16.0376</v>
       </c>
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="n">
         <v>65</v>
       </c>
       <c r="AT2" t="n">
-        <v>72</v>
+        <v>72.5</v>
       </c>
       <c r="AU2" t="n">
         <v>49.5</v>
       </c>
       <c r="AV2" t="n">
-        <v>77.40000000000001</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="AW2" t="n">
         <v>757</v>
       </c>
       <c r="AX2" t="n">
-        <v>17.838</v>
+        <v>17.874</v>
       </c>
       <c r="AY2" t="n">
         <v>18.81</v>
       </c>
       <c r="AZ2" t="n">
-        <v>-1.6</v>
+        <v>-1.4</v>
       </c>
       <c r="BA2" t="n">
-        <v>11.23</v>
+        <v>11.45</v>
       </c>
       <c r="BB2" t="inlineStr"/>
       <c r="BC2" t="inlineStr"/>
@@ -972,24 +972,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>SMH</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>NVIDIA Corporation</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
+          <t>VanEck Semiconductor ETF</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>69.90000000000001</v>
+        <v>57.7</v>
       </c>
       <c r="F3" t="n">
-        <v>51.7</v>
+        <v>48</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -1003,7 +999,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>score 69.9; priority 51.7; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 57.7; priority 48.0; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1018,22 +1014,22 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma</t>
+          <t>prezzo 4.1% sotto MA50: attendere recupero</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>NVDA: scenario base Accumulate Carefully, score 69.9, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -0.7%.</t>
+          <t>SMH: scenario base Hold / Monitor, score 57.7, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -4.1%.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 230.10 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 668.91 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 189.80 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 504.22 o peggioramento trend; rischio attuale: High risk.</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -1043,7 +1039,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Accumulate Carefully</t>
+          <t>Hold / Monitor</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -1052,149 +1048,127 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>189.7976</v>
+        <v>504.22</v>
       </c>
       <c r="T3" t="n">
-        <v>230.1025</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>NVIDIA Corporation</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
+        <v>668.91</v>
+      </c>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>VanEck Semiconductor ETF</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Thematic</t>
+        </is>
+      </c>
       <c r="X3" t="inlineStr">
         <is>
           <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y3" t="n">
-        <v>3.02</v>
+        <v>-12.12</v>
       </c>
       <c r="Z3" t="n">
-        <v>19.47</v>
+        <v>79.81999999999999</v>
       </c>
       <c r="AA3" t="n">
-        <v>46.98</v>
+        <v>37.04</v>
       </c>
       <c r="AB3" t="n">
-        <v>-36.88</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>26.73</v>
-      </c>
-      <c r="AD3" t="n">
-        <v>13.53</v>
-      </c>
+        <v>-35.74</v>
+      </c>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
-        </is>
-      </c>
-      <c r="AF3" t="inlineStr"/>
+          <t>Rischio elevato: usare solo come quota satellite e con size ridotta.</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>Semiconduttori</t>
+        </is>
+      </c>
       <c r="AG3" t="n">
-        <v>211.16</v>
-      </c>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
+        <v>544.83</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>22</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>73.59999999999999</v>
+      </c>
       <c r="AL3" t="n">
-        <v>-6.17</v>
+        <v>-7.52</v>
       </c>
       <c r="AM3" t="n">
-        <v>17.42</v>
+        <v>40.66</v>
       </c>
       <c r="AN3" t="n">
-        <v>67.31999999999999</v>
+        <v>54.29</v>
       </c>
       <c r="AO3" t="n">
-        <v>1.43</v>
+        <v>1.47</v>
       </c>
       <c r="AP3" t="n">
-        <v>212.6871</v>
+        <v>568.1546</v>
       </c>
       <c r="AQ3" t="n">
-        <v>197.2504</v>
+        <v>483.089</v>
       </c>
       <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="n">
         <v>65</v>
       </c>
       <c r="AT3" t="n">
-        <v>69.59999999999999</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="AU3" t="n">
-        <v>14.1</v>
+        <v>27</v>
       </c>
       <c r="AV3" t="n">
-        <v>78.7</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="AW3" t="n">
         <v>752</v>
       </c>
       <c r="AX3" t="n">
-        <v>208.247</v>
+        <v>544.83</v>
       </c>
       <c r="AY3" t="n">
-        <v>230.1025</v>
+        <v>594.0700000000001</v>
       </c>
       <c r="AZ3" t="n">
-        <v>-0.72</v>
+        <v>-4.11</v>
       </c>
       <c r="BA3" t="n">
-        <v>7.05</v>
-      </c>
-      <c r="BB3" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="BC3" t="inlineStr">
-        <is>
-          <t>Semiconductors</t>
-        </is>
-      </c>
-      <c r="BD3" t="n">
-        <v>5099725783040</v>
-      </c>
-      <c r="BE3" t="n">
-        <v>63.66</v>
-      </c>
-      <c r="BF3" t="n">
-        <v>117.21</v>
-      </c>
-      <c r="BG3" t="n">
-        <v>105.9</v>
-      </c>
-      <c r="BH3" t="n">
-        <v>16.97</v>
-      </c>
-      <c r="BI3" t="n">
-        <v>46</v>
-      </c>
-      <c r="BJ3" t="n">
-        <v>100</v>
-      </c>
-      <c r="BK3" t="n">
-        <v>69.59999999999999</v>
-      </c>
-      <c r="BL3" t="n">
-        <v>77.8</v>
-      </c>
-      <c r="BM3" t="n">
-        <v>14.1</v>
-      </c>
-      <c r="BN3" t="n">
-        <v>78.7</v>
-      </c>
+        <v>12.78</v>
+      </c>
+      <c r="BB3" t="inlineStr"/>
+      <c r="BC3" t="inlineStr"/>
+      <c r="BD3" t="inlineStr"/>
+      <c r="BE3" t="inlineStr"/>
+      <c r="BF3" t="inlineStr"/>
+      <c r="BG3" t="inlineStr"/>
+      <c r="BH3" t="inlineStr"/>
+      <c r="BI3" t="inlineStr"/>
+      <c r="BJ3" t="inlineStr"/>
+      <c r="BK3" t="inlineStr"/>
+      <c r="BL3" t="inlineStr"/>
+      <c r="BM3" t="inlineStr"/>
+      <c r="BN3" t="inlineStr"/>
       <c r="BO3" t="inlineStr"/>
-      <c r="BP3" t="inlineStr">
-        <is>
-          <t>USA / Semiconductors</t>
-        </is>
-      </c>
+      <c r="BP3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1214,10 +1188,10 @@
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>58.3</v>
+        <v>57.2</v>
       </c>
       <c r="F4" t="n">
-        <v>50.9</v>
+        <v>47</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1231,7 +1205,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>score 58.3; priority 50.9; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 57.2; priority 47.0; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1251,7 +1225,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>WCLD.MI: scenario base Hold / Monitor, score 58.3, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 5.9%.</t>
+          <t>WCLD.MI: scenario base Hold / Monitor, score 57.2, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 7.8%.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -1302,13 +1276,13 @@
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>31.99</v>
+        <v>34.47</v>
       </c>
       <c r="Z4" t="n">
-        <v>13.72</v>
+        <v>15.85</v>
       </c>
       <c r="AA4" t="n">
-        <v>35.19</v>
+        <v>35.29</v>
       </c>
       <c r="AB4" t="n">
         <v>-48.6</v>
@@ -1326,37 +1300,37 @@
         </is>
       </c>
       <c r="AG4" t="n">
-        <v>34.16</v>
+        <v>34.8</v>
       </c>
       <c r="AH4" t="n">
-        <v>26</v>
+        <v>26.3</v>
       </c>
       <c r="AI4" t="n">
         <v>100</v>
       </c>
       <c r="AJ4" t="n">
-        <v>13.9</v>
+        <v>13.8</v>
       </c>
       <c r="AK4" t="n">
-        <v>75.3</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="AL4" t="n">
-        <v>-1.6</v>
+        <v>0.24</v>
       </c>
       <c r="AM4" t="n">
-        <v>39.6</v>
+        <v>42.21</v>
       </c>
       <c r="AN4" t="n">
-        <v>6.1</v>
+        <v>6.76</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.17</v>
+        <v>0.19</v>
       </c>
       <c r="AP4" t="n">
-        <v>32.27</v>
+        <v>32.2828</v>
       </c>
       <c r="AQ4" t="n">
-        <v>27.2767</v>
+        <v>27.2799</v>
       </c>
       <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="n">
@@ -1366,10 +1340,10 @@
         <v>100</v>
       </c>
       <c r="AU4" t="n">
-        <v>18.9</v>
+        <v>18.8</v>
       </c>
       <c r="AV4" t="n">
-        <v>75.3</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="AW4" t="n">
         <v>758</v>
@@ -1381,10 +1355,10 @@
         <v>36.89</v>
       </c>
       <c r="AZ4" t="n">
-        <v>5.86</v>
+        <v>7.8</v>
       </c>
       <c r="BA4" t="n">
-        <v>25.24</v>
+        <v>27.57</v>
       </c>
       <c r="BB4" t="inlineStr"/>
       <c r="BC4" t="inlineStr"/>
@@ -1410,20 +1384,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SMH</t>
+          <t>INRG.MI</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>VanEck Semiconductor ETF</t>
+          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>57.5</v>
+        <v>39.7</v>
       </c>
       <c r="F5" t="n">
-        <v>47.8</v>
+        <v>46.6</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1437,37 +1411,37 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>score 57.5; priority 47.8; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 39.7; priority 46.6; trend: Weak; entry zone: Wait for trend repair; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Monitor / partial entry only</t>
+          <t>Wait for trend repair</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>High risk</t>
+          <t>Medium-high risk</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>prezzo 4.3% sotto MA50: attendere recupero</t>
+          <t>prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>SMH: scenario base Hold / Monitor, score 57.5, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -4.3%.</t>
+          <t>INRG.MI: scenario base Avoid for Now, score 39.7, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -3.0%.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 668.91 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 10.53 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 504.22 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 8.54 o peggioramento trend; rischio attuale: Medium-high risk.</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -1477,24 +1451,24 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Hold / Monitor</t>
+          <t>Avoid for Now</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Constructive</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="S5" t="n">
-        <v>504.22</v>
+        <v>8.541</v>
       </c>
       <c r="T5" t="n">
-        <v>668.91</v>
+        <v>10.53</v>
       </c>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>VanEck Semiconductor ETF</t>
+          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
@@ -1508,16 +1482,16 @@
         </is>
       </c>
       <c r="Y5" t="n">
-        <v>-12.26</v>
+        <v>-15.36</v>
       </c>
       <c r="Z5" t="n">
-        <v>79.53</v>
+        <v>21.88</v>
       </c>
       <c r="AA5" t="n">
-        <v>37.05</v>
+        <v>24.21</v>
       </c>
       <c r="AB5" t="n">
-        <v>-35.74</v>
+        <v>-34.52</v>
       </c>
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
@@ -1528,69 +1502,69 @@
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>Semiconduttori</t>
+          <t>Energia pulita</t>
         </is>
       </c>
       <c r="AG5" t="n">
-        <v>543.95</v>
+        <v>8.753</v>
       </c>
       <c r="AH5" t="n">
-        <v>52.5</v>
+        <v>34.2</v>
       </c>
       <c r="AI5" t="n">
-        <v>77</v>
+        <v>30.4</v>
       </c>
       <c r="AJ5" t="n">
-        <v>22</v>
+        <v>38.3</v>
       </c>
       <c r="AK5" t="n">
-        <v>73.40000000000001</v>
+        <v>70.8</v>
       </c>
       <c r="AL5" t="n">
-        <v>-7.67</v>
+        <v>-3.52</v>
       </c>
       <c r="AM5" t="n">
-        <v>40.44</v>
+        <v>-5.93</v>
       </c>
       <c r="AN5" t="n">
-        <v>54.21</v>
+        <v>2.08</v>
       </c>
       <c r="AO5" t="n">
-        <v>1.46</v>
+        <v>0.09</v>
       </c>
       <c r="AP5" t="n">
-        <v>568.1369999999999</v>
+        <v>9.023300000000001</v>
       </c>
       <c r="AQ5" t="n">
-        <v>483.0846</v>
+        <v>9.3093</v>
       </c>
       <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="n">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="AT5" t="n">
-        <v>77</v>
+        <v>30.4</v>
       </c>
       <c r="AU5" t="n">
-        <v>27</v>
+        <v>43.3</v>
       </c>
       <c r="AV5" t="n">
-        <v>73.40000000000001</v>
+        <v>70.8</v>
       </c>
       <c r="AW5" t="n">
-        <v>752</v>
+        <v>757</v>
       </c>
       <c r="AX5" t="n">
-        <v>543.95</v>
+        <v>8.541</v>
       </c>
       <c r="AY5" t="n">
-        <v>594.0700000000001</v>
+        <v>9.073</v>
       </c>
       <c r="AZ5" t="n">
-        <v>-4.26</v>
+        <v>-3</v>
       </c>
       <c r="BA5" t="n">
-        <v>12.6</v>
+        <v>-5.98</v>
       </c>
       <c r="BB5" t="inlineStr"/>
       <c r="BC5" t="inlineStr"/>
@@ -1616,20 +1590,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>INRG.MI</t>
+          <t>ASML.AS</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>ASML Holding N.V.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
       <c r="E6" t="n">
-        <v>39.8</v>
+        <v>58.8</v>
       </c>
       <c r="F6" t="n">
-        <v>46.8</v>
+        <v>43.6</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1643,37 +1621,37 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>score 39.8; priority 46.8; trend: Weak; entry zone: Wait for trend repair; risk flag: Medium-high risk</t>
+          <t>score 58.8; priority 43.6; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Wait for trend repair</t>
+          <t>Monitor / partial entry only</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Medium-high risk</t>
+          <t>High risk</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo 8.0% sotto MA50: attendere recupero; vicino a supporto 60D: controllare tenuta e volumi</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>INRG.MI: scenario base Avoid for Now, score 39.8, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -2.8%.</t>
+          <t>ASML.AS: scenario base Hold / Monitor, score 58.8, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -8.0%.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 10.53 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 1719.33 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 8.54 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+          <t>Scenario negativo: perdita area 1362.20 o peggioramento trend; rischio attuale: High risk.</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -1683,136 +1661,158 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Avoid for Now</t>
+          <t>Hold / Monitor</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Constructive</t>
         </is>
       </c>
       <c r="S6" t="n">
-        <v>8.541</v>
+        <v>1362.2</v>
       </c>
       <c r="T6" t="n">
-        <v>10.53</v>
-      </c>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>Thematic</t>
-        </is>
-      </c>
+        <v>1719.3295</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>ASML Holding N.V.</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr">
         <is>
           <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y6" t="n">
-        <v>-15.15</v>
+        <v>-12.68</v>
       </c>
       <c r="Z6" t="n">
-        <v>22.18</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="AA6" t="n">
-        <v>24.21</v>
+        <v>39.74</v>
       </c>
       <c r="AB6" t="n">
-        <v>-34.52</v>
-      </c>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
+        <v>-44.77</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>54.57</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>26.83</v>
+      </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>Rischio elevato: usare solo come quota satellite e con size ridotta.</t>
-        </is>
-      </c>
-      <c r="AF6" t="inlineStr">
-        <is>
-          <t>Energia pulita</t>
-        </is>
-      </c>
+          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="n">
-        <v>8.775</v>
-      </c>
-      <c r="AH6" t="n">
-        <v>34.2</v>
-      </c>
-      <c r="AI6" t="n">
-        <v>30.9</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>71.09999999999999</v>
-      </c>
+        <v>1387.8</v>
+      </c>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
       <c r="AL6" t="n">
-        <v>-3.27</v>
+        <v>-13.77</v>
       </c>
       <c r="AM6" t="n">
-        <v>-5.69</v>
+        <v>16.3</v>
       </c>
       <c r="AN6" t="n">
-        <v>2.17</v>
+        <v>34.3</v>
       </c>
       <c r="AO6" t="n">
-        <v>0.09</v>
+        <v>0.86</v>
       </c>
       <c r="AP6" t="n">
-        <v>9.0237</v>
+        <v>1507.9715</v>
       </c>
       <c r="AQ6" t="n">
-        <v>9.3094</v>
+        <v>1295.8383</v>
       </c>
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="n">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="AT6" t="n">
-        <v>30.9</v>
+        <v>64.7</v>
       </c>
       <c r="AU6" t="n">
-        <v>43.3</v>
+        <v>16.5</v>
       </c>
       <c r="AV6" t="n">
-        <v>71.09999999999999</v>
+        <v>67.8</v>
       </c>
       <c r="AW6" t="n">
-        <v>757</v>
+        <v>764</v>
       </c>
       <c r="AX6" t="n">
-        <v>8.541</v>
+        <v>1387.8</v>
       </c>
       <c r="AY6" t="n">
-        <v>9.073</v>
+        <v>1621.2</v>
       </c>
       <c r="AZ6" t="n">
-        <v>-2.76</v>
+        <v>-7.97</v>
       </c>
       <c r="BA6" t="n">
-        <v>-5.74</v>
-      </c>
-      <c r="BB6" t="inlineStr"/>
-      <c r="BC6" t="inlineStr"/>
-      <c r="BD6" t="inlineStr"/>
-      <c r="BE6" t="inlineStr"/>
-      <c r="BF6" t="inlineStr"/>
-      <c r="BG6" t="inlineStr"/>
-      <c r="BH6" t="inlineStr"/>
-      <c r="BI6" t="inlineStr"/>
-      <c r="BJ6" t="inlineStr"/>
-      <c r="BK6" t="inlineStr"/>
-      <c r="BL6" t="inlineStr"/>
-      <c r="BM6" t="inlineStr"/>
-      <c r="BN6" t="inlineStr"/>
+        <v>7.1</v>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="BC6" t="inlineStr">
+        <is>
+          <t>Semiconductor Equipment &amp; Materials</t>
+        </is>
+      </c>
+      <c r="BD6" t="n">
+        <v>533053997056</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>30.11</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>53.94</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>9.09</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>53</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>100</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="BN6" t="n">
+        <v>67.8</v>
+      </c>
       <c r="BO6" t="inlineStr"/>
-      <c r="BP6" t="inlineStr"/>
+      <c r="BP6" t="inlineStr">
+        <is>
+          <t>Europe / Semiconductors</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1822,12 +1822,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ASML.AS</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ASML Holding N.V.</t>
+          <t>Tesla, Inc.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1836,10 +1836,10 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>58.7</v>
+        <v>35.7</v>
       </c>
       <c r="F7" t="n">
-        <v>43.4</v>
+        <v>28.2</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1853,7 +1853,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>score 58.7; priority 43.4; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 35.7; priority 28.2; trend: Recovery; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1868,22 +1868,22 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>prezzo 8.1% sotto MA50: attendere recupero; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>ASML.AS: scenario base Hold / Monitor, score 58.7, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -8.1%.</t>
+          <t>TSLA: scenario base High Risk, score 35.7, trend Recovery. Entry zone: Monitor / partial entry only. Distanza da MA50: 2.8%.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 1719.33 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 425.30 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 1362.20 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 298.32 o peggioramento trend; rischio attuale: High risk.</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1893,23 +1893,23 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Hold / Monitor</t>
+          <t>High Risk</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Constructive</t>
+          <t>Recovery</t>
         </is>
       </c>
       <c r="S7" t="n">
-        <v>1362.2</v>
+        <v>298.32</v>
       </c>
       <c r="T7" t="n">
-        <v>1719.3295</v>
+        <v>425.3</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>ASML Holding N.V.</t>
+          <t>Tesla, Inc.</t>
         </is>
       </c>
       <c r="V7" t="inlineStr"/>
@@ -1920,22 +1920,22 @@
         </is>
       </c>
       <c r="Y7" t="n">
-        <v>-12.83</v>
+        <v>-10.51</v>
       </c>
       <c r="Z7" t="n">
-        <v>90.27</v>
+        <v>-1.39</v>
       </c>
       <c r="AA7" t="n">
-        <v>39.75</v>
+        <v>58.18</v>
       </c>
       <c r="AB7" t="n">
-        <v>-44.77</v>
+        <v>-53.77</v>
       </c>
       <c r="AC7" t="n">
-        <v>54.47</v>
+        <v>330.62</v>
       </c>
       <c r="AD7" t="n">
-        <v>26.78</v>
+        <v>168.48</v>
       </c>
       <c r="AE7" t="inlineStr">
         <is>
@@ -1944,158 +1944,152 @@
       </c>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="n">
-        <v>1385.4</v>
+        <v>363.6999</v>
       </c>
       <c r="AH7" t="inlineStr"/>
       <c r="AI7" t="inlineStr"/>
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr"/>
       <c r="AL7" t="n">
-        <v>-13.92</v>
+        <v>6.98</v>
       </c>
       <c r="AM7" t="n">
-        <v>16.1</v>
+        <v>-7.03</v>
       </c>
       <c r="AN7" t="n">
-        <v>34.22</v>
+        <v>9.68</v>
       </c>
       <c r="AO7" t="n">
-        <v>0.86</v>
+        <v>0.17</v>
       </c>
       <c r="AP7" t="n">
-        <v>1507.9235</v>
+        <v>353.9032</v>
       </c>
       <c r="AQ7" t="n">
-        <v>1295.8263</v>
+        <v>398.6551</v>
       </c>
       <c r="AR7" t="inlineStr"/>
       <c r="AS7" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="AT7" t="n">
-        <v>64.3</v>
+        <v>30.7</v>
       </c>
       <c r="AU7" t="n">
-        <v>16.5</v>
+        <v>0</v>
       </c>
       <c r="AV7" t="n">
-        <v>67.59999999999999</v>
+        <v>78.2</v>
       </c>
       <c r="AW7" t="n">
-        <v>764</v>
+        <v>752</v>
       </c>
       <c r="AX7" t="n">
-        <v>1385.2</v>
+        <v>336.87</v>
       </c>
       <c r="AY7" t="n">
-        <v>1621.2</v>
+        <v>376.37</v>
       </c>
       <c r="AZ7" t="n">
-        <v>-8.140000000000001</v>
+        <v>2.76</v>
       </c>
       <c r="BA7" t="n">
-        <v>6.9</v>
+        <v>-8.77</v>
       </c>
       <c r="BB7" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="BC7" t="inlineStr">
         <is>
-          <t>Semiconductor Equipment &amp; Materials</t>
+          <t>Auto Manufacturers</t>
         </is>
       </c>
       <c r="BD7" t="n">
-        <v>532055293952</v>
+        <v>1436371386368</v>
       </c>
       <c r="BE7" t="n">
-        <v>30.11</v>
+        <v>3.67</v>
       </c>
       <c r="BF7" t="n">
-        <v>53.94</v>
+        <v>4.67</v>
       </c>
       <c r="BG7" t="n">
-        <v>21.3</v>
+        <v>25.5</v>
       </c>
       <c r="BH7" t="n">
-        <v>9.09</v>
-      </c>
-      <c r="BI7" t="n">
-        <v>53</v>
-      </c>
+        <v>18.37</v>
+      </c>
+      <c r="BI7" t="inlineStr"/>
       <c r="BJ7" t="n">
-        <v>100</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="BK7" t="n">
-        <v>64.3</v>
+        <v>30.7</v>
       </c>
       <c r="BL7" t="n">
-        <v>26.6</v>
+        <v>0</v>
       </c>
       <c r="BM7" t="n">
-        <v>16.5</v>
+        <v>0</v>
       </c>
       <c r="BN7" t="n">
-        <v>67.59999999999999</v>
+        <v>78.2</v>
       </c>
       <c r="BO7" t="inlineStr"/>
       <c r="BP7" t="inlineStr">
         <is>
-          <t>Europe / Semiconductors</t>
+          <t>USA / EV</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2. Rischio da controllare</t>
+          <t>1. Da guardare oggi</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>XDEV.MI</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tesla, Inc.</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
+          <t>Xtrackers MSCI World Value UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>35.3</v>
+        <v>79.2</v>
       </c>
       <c r="F8" t="n">
-        <v>27.8</v>
+        <v>79.3</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>🟥 Riduci rischio / non aumentare</t>
+          <t>🟢 Valuta ingresso graduale</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Non aumentare esposizione: controlla peso in portafoglio, stop mentale e correlazione con posizioni simili.</t>
+          <t>Non entrare a mercato alla cieca: valuta ingresso graduale, size piccola e conferma su trend/supporti.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>score 35.3; priority 27.8; trend: Recovery; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 79.2; priority 79.3; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Monitor / partial entry only</t>
+          <t>Constructive entry zone</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>High risk</t>
+          <t>Normal risk</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -2105,17 +2099,17 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>TSLA: scenario base High Risk, score 35.3, trend Recovery. Entry zone: Monitor / partial entry only. Distanza da MA50: 1.9%.</t>
+          <t>XDEV.MI: scenario base Buy Watchlist, score 79.2, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 2.1%.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 425.30 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 74.49 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 298.32 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 69.45 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -2125,223 +2119,207 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>High Risk</t>
+          <t>Buy Watchlist</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Recovery</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="S8" t="n">
-        <v>298.32</v>
+        <v>69.45</v>
       </c>
       <c r="T8" t="n">
-        <v>425.3</v>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>Tesla, Inc.</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
+        <v>74.48999999999999</v>
+      </c>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI World Value UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>Ridurre size / solo monitoraggio</t>
+          <t>Priorità watchlist</t>
         </is>
       </c>
       <c r="Y8" t="n">
-        <v>-11.33</v>
+        <v>2.44</v>
       </c>
       <c r="Z8" t="n">
-        <v>-2.28</v>
+        <v>54.67</v>
       </c>
       <c r="AA8" t="n">
-        <v>58.19</v>
+        <v>14.15</v>
       </c>
       <c r="AB8" t="n">
-        <v>-53.77</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>327.68</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>166.98</v>
-      </c>
+        <v>-17.8</v>
+      </c>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
-        </is>
-      </c>
-      <c r="AF8" t="inlineStr"/>
+          <t>ETF forte e in trend favorevole; valutare solo con coerenza di portafoglio.</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>Value globale</t>
+        </is>
+      </c>
       <c r="AG8" t="n">
-        <v>360.4</v>
-      </c>
-      <c r="AH8" t="inlineStr"/>
-      <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr"/>
+        <v>73.47</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>84.40000000000001</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>82.8</v>
+      </c>
       <c r="AL8" t="n">
-        <v>6.01</v>
+        <v>0.29</v>
       </c>
       <c r="AM8" t="n">
-        <v>-7.87</v>
+        <v>28.8</v>
       </c>
       <c r="AN8" t="n">
-        <v>9.35</v>
+        <v>25.21</v>
       </c>
       <c r="AO8" t="n">
-        <v>0.16</v>
+        <v>1.78</v>
       </c>
       <c r="AP8" t="n">
-        <v>353.8372</v>
+        <v>71.961</v>
       </c>
       <c r="AQ8" t="n">
-        <v>398.6386</v>
+        <v>62.9354</v>
       </c>
       <c r="AR8" t="inlineStr"/>
       <c r="AS8" t="n">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="AT8" t="n">
-        <v>28.9</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="AU8" t="n">
-        <v>0</v>
+        <v>68.8</v>
       </c>
       <c r="AV8" t="n">
-        <v>78.2</v>
+        <v>82.8</v>
       </c>
       <c r="AW8" t="n">
-        <v>752</v>
+        <v>757</v>
       </c>
       <c r="AX8" t="n">
-        <v>336.87</v>
+        <v>71.86</v>
       </c>
       <c r="AY8" t="n">
-        <v>376.37</v>
+        <v>74.48999999999999</v>
       </c>
       <c r="AZ8" t="n">
-        <v>1.85</v>
+        <v>2.1</v>
       </c>
       <c r="BA8" t="n">
-        <v>-9.59</v>
-      </c>
-      <c r="BB8" t="inlineStr">
-        <is>
-          <t>Consumer Cyclical</t>
-        </is>
-      </c>
-      <c r="BC8" t="inlineStr">
-        <is>
-          <t>Auto Manufacturers</t>
-        </is>
-      </c>
-      <c r="BD8" t="n">
-        <v>1423613231104</v>
-      </c>
-      <c r="BE8" t="n">
-        <v>3.67</v>
-      </c>
-      <c r="BF8" t="n">
-        <v>4.67</v>
-      </c>
-      <c r="BG8" t="n">
-        <v>25.5</v>
-      </c>
-      <c r="BH8" t="n">
-        <v>18.37</v>
-      </c>
+        <v>16.74</v>
+      </c>
+      <c r="BB8" t="inlineStr"/>
+      <c r="BC8" t="inlineStr"/>
+      <c r="BD8" t="inlineStr"/>
+      <c r="BE8" t="inlineStr"/>
+      <c r="BF8" t="inlineStr"/>
+      <c r="BG8" t="inlineStr"/>
+      <c r="BH8" t="inlineStr"/>
       <c r="BI8" t="inlineStr"/>
-      <c r="BJ8" t="n">
-        <v>69.90000000000001</v>
-      </c>
-      <c r="BK8" t="n">
-        <v>28.9</v>
-      </c>
-      <c r="BL8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN8" t="n">
-        <v>78.2</v>
-      </c>
+      <c r="BJ8" t="inlineStr"/>
+      <c r="BK8" t="inlineStr"/>
+      <c r="BL8" t="inlineStr"/>
+      <c r="BM8" t="inlineStr"/>
+      <c r="BN8" t="inlineStr"/>
       <c r="BO8" t="inlineStr"/>
-      <c r="BP8" t="inlineStr">
-        <is>
-          <t>USA / EV</t>
-        </is>
-      </c>
+      <c r="BP8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1. Da guardare oggi</t>
+          <t>3. Interessanti ma da attendere</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>XDEV.MI</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Value UCITS ETF 1C</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
       <c r="E9" t="n">
-        <v>79.2</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>79.3</v>
+        <v>63</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>🟢 Valuta ingresso graduale</t>
+          <t>🟠 Attendi pullback</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Non entrare a mercato alla cieca: valuta ingresso graduale, size piccola e conferma su trend/supporti.</t>
+          <t>Non inseguire il prezzo: imposta alert su pullback o tenuta supporto. Supporto 60D: 352.167.</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>score 79.2; priority 79.3; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 78.4; priority 63.0; trend: Bullish; entry zone: Extended - wait pullback; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Constructive entry zone</t>
+          <t>Extended - wait pullback</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Normal risk</t>
+          <t>Medium-high risk</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma</t>
+          <t>prezzo 11.0% sopra MA50: evitare inseguimento</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>XDEV.MI: scenario base Buy Watchlist, score 79.2, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 2.1%.</t>
+          <t>MSFT: scenario base Buy Watchlist, score 78.4, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 11.0%.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 74.49 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 513.53 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 69.45 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 352.17 o peggioramento trend; rischio attuale: Medium-high risk.</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -2360,127 +2338,149 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>69.45</v>
+        <v>352.167</v>
       </c>
       <c r="T9" t="n">
-        <v>74.48999999999999</v>
-      </c>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>Xtrackers MSCI World Value UCITS ETF 1C</t>
-        </is>
-      </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>Factor</t>
-        </is>
-      </c>
+        <v>513.53</v>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr">
         <is>
-          <t>Priorità watchlist</t>
+          <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y9" t="n">
-        <v>2.45</v>
+        <v>29.56</v>
       </c>
       <c r="Z9" t="n">
-        <v>54.69</v>
+        <v>1.69</v>
       </c>
       <c r="AA9" t="n">
-        <v>14.15</v>
+        <v>26.25</v>
       </c>
       <c r="AB9" t="n">
-        <v>-17.8</v>
-      </c>
-      <c r="AC9" t="inlineStr"/>
-      <c r="AD9" t="inlineStr"/>
+        <v>-34.5</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>28.17</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>21.44</v>
+      </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>ETF forte e in trend favorevole; valutare solo con coerenza di portafoglio.</t>
-        </is>
-      </c>
-      <c r="AF9" t="inlineStr">
-        <is>
-          <t>Value globale</t>
-        </is>
-      </c>
+          <t>Titolo forte; resta necessario controllare prezzo, trimestrali e size.</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="n">
-        <v>73.48</v>
-      </c>
-      <c r="AH9" t="n">
-        <v>76.7</v>
-      </c>
-      <c r="AI9" t="n">
-        <v>84.40000000000001</v>
-      </c>
-      <c r="AJ9" t="n">
-        <v>68.8</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>82.8</v>
-      </c>
+        <v>505.305</v>
+      </c>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
       <c r="AL9" t="n">
-        <v>0.3</v>
+        <v>1.89</v>
       </c>
       <c r="AM9" t="n">
-        <v>28.82</v>
+        <v>28.27</v>
       </c>
       <c r="AN9" t="n">
-        <v>25.21</v>
+        <v>15.24</v>
       </c>
       <c r="AO9" t="n">
-        <v>1.78</v>
+        <v>0.58</v>
       </c>
       <c r="AP9" t="n">
-        <v>71.96120000000001</v>
+        <v>455.426</v>
       </c>
       <c r="AQ9" t="n">
-        <v>62.9355</v>
+        <v>429.8254</v>
       </c>
       <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="n">
         <v>85</v>
       </c>
       <c r="AT9" t="n">
-        <v>84.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="AU9" t="n">
-        <v>68.8</v>
+        <v>40.9</v>
       </c>
       <c r="AV9" t="n">
-        <v>82.8</v>
+        <v>54.9</v>
       </c>
       <c r="AW9" t="n">
-        <v>757</v>
+        <v>752</v>
       </c>
       <c r="AX9" t="n">
-        <v>71.86</v>
+        <v>479.4474</v>
       </c>
       <c r="AY9" t="n">
-        <v>74.48999999999999</v>
+        <v>513.53</v>
       </c>
       <c r="AZ9" t="n">
-        <v>2.11</v>
+        <v>10.96</v>
       </c>
       <c r="BA9" t="n">
-        <v>16.75</v>
-      </c>
-      <c r="BB9" t="inlineStr"/>
-      <c r="BC9" t="inlineStr"/>
-      <c r="BD9" t="inlineStr"/>
-      <c r="BE9" t="inlineStr"/>
-      <c r="BF9" t="inlineStr"/>
-      <c r="BG9" t="inlineStr"/>
-      <c r="BH9" t="inlineStr"/>
-      <c r="BI9" t="inlineStr"/>
-      <c r="BJ9" t="inlineStr"/>
-      <c r="BK9" t="inlineStr"/>
-      <c r="BL9" t="inlineStr"/>
-      <c r="BM9" t="inlineStr"/>
-      <c r="BN9" t="inlineStr"/>
+        <v>17.57</v>
+      </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="BC9" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+      <c r="BD9" t="n">
+        <v>3752499609600</v>
+      </c>
+      <c r="BE9" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>34.04</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>29.12</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>73</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>100</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>100</v>
+      </c>
+      <c r="BL9" t="n">
+        <v>64.90000000000001</v>
+      </c>
+      <c r="BM9" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="BN9" t="n">
+        <v>54.9</v>
+      </c>
       <c r="BO9" t="inlineStr"/>
-      <c r="BP9" t="inlineStr"/>
+      <c r="BP9" t="inlineStr">
+        <is>
+          <t>USA / Technology</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2504,10 +2504,10 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>75.2</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>74.7</v>
+        <v>74.5</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>score 75.2; priority 74.7; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 75.1; priority 74.5; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>AAPL: scenario base Accumulate Carefully, score 75.2, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 5.0%.</t>
+          <t>AAPL: scenario base Accumulate Carefully, score 75.1, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 5.2%.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -2588,10 +2588,10 @@
         </is>
       </c>
       <c r="Y10" t="n">
-        <v>14.87</v>
+        <v>15.09</v>
       </c>
       <c r="Z10" t="n">
-        <v>45.8</v>
+        <v>46.08</v>
       </c>
       <c r="AA10" t="n">
         <v>26.86</v>
@@ -2600,10 +2600,10 @@
         <v>-33.36</v>
       </c>
       <c r="AC10" t="n">
-        <v>38.36</v>
+        <v>38.44</v>
       </c>
       <c r="AD10" t="n">
-        <v>34.87</v>
+        <v>34.94</v>
       </c>
       <c r="AE10" t="inlineStr">
         <is>
@@ -2612,29 +2612,29 @@
       </c>
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="n">
-        <v>334.145</v>
+        <v>334.78</v>
       </c>
       <c r="AH10" t="inlineStr"/>
       <c r="AI10" t="inlineStr"/>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
       <c r="AL10" t="n">
-        <v>9.460000000000001</v>
+        <v>9.67</v>
       </c>
       <c r="AM10" t="n">
-        <v>33.83</v>
+        <v>34.09</v>
       </c>
       <c r="AN10" t="n">
-        <v>24.59</v>
+        <v>24.67</v>
       </c>
       <c r="AO10" t="n">
         <v>0.92</v>
       </c>
       <c r="AP10" t="n">
-        <v>318.346</v>
+        <v>318.3587</v>
       </c>
       <c r="AQ10" t="n">
-        <v>284.8318</v>
+        <v>284.8349</v>
       </c>
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="n">
@@ -2647,7 +2647,7 @@
         <v>41.1</v>
       </c>
       <c r="AV10" t="n">
-        <v>78.90000000000001</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="AW10" t="n">
         <v>752</v>
@@ -2656,13 +2656,13 @@
         <v>305.59</v>
       </c>
       <c r="AY10" t="n">
-        <v>334.13</v>
+        <v>334.78</v>
       </c>
       <c r="AZ10" t="n">
-        <v>4.96</v>
+        <v>5.16</v>
       </c>
       <c r="BA10" t="n">
-        <v>17.31</v>
+        <v>17.53</v>
       </c>
       <c r="BB10" t="inlineStr">
         <is>
@@ -2675,7 +2675,7 @@
         </is>
       </c>
       <c r="BD10" t="n">
-        <v>4876280528896</v>
+        <v>4885839347712</v>
       </c>
       <c r="BE10" t="n">
         <v>27.62</v>
@@ -2699,13 +2699,13 @@
         <v>100</v>
       </c>
       <c r="BL10" t="n">
-        <v>33.8</v>
+        <v>33.6</v>
       </c>
       <c r="BM10" t="n">
         <v>41.1</v>
       </c>
       <c r="BN10" t="n">
-        <v>78.90000000000001</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="BO10" t="inlineStr"/>
       <c r="BP10" t="inlineStr">
@@ -2732,10 +2732,10 @@
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>72</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>74.09999999999999</v>
+        <v>74</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -2749,7 +2749,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>score 72.0; priority 74.1; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 71.9; priority 74.0; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>MVOL.MI: scenario base Accumulate Carefully, score 72.0, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.1%.</t>
+          <t>MVOL.MI: scenario base Accumulate Carefully, score 71.9, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.9%.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -2820,13 +2820,13 @@
         </is>
       </c>
       <c r="Y11" t="n">
-        <v>5.72</v>
+        <v>5.51</v>
       </c>
       <c r="Z11" t="n">
-        <v>7.26</v>
+        <v>7.06</v>
       </c>
       <c r="AA11" t="n">
-        <v>9.710000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="AB11" t="n">
         <v>-12.85</v>
@@ -2844,13 +2844,13 @@
         </is>
       </c>
       <c r="AG11" t="n">
-        <v>67.5</v>
+        <v>67.37</v>
       </c>
       <c r="AH11" t="n">
         <v>62.9</v>
       </c>
       <c r="AI11" t="n">
-        <v>61.9</v>
+        <v>61.4</v>
       </c>
       <c r="AJ11" t="n">
         <v>78.09999999999999</v>
@@ -2859,29 +2859,29 @@
         <v>82.8</v>
       </c>
       <c r="AL11" t="n">
-        <v>-0.03</v>
+        <v>-0.22</v>
       </c>
       <c r="AM11" t="n">
-        <v>3.45</v>
+        <v>3.25</v>
       </c>
       <c r="AN11" t="n">
-        <v>7.61</v>
+        <v>7.54</v>
       </c>
       <c r="AO11" t="n">
         <v>0.78</v>
       </c>
       <c r="AP11" t="n">
-        <v>66.7974</v>
+        <v>66.7948</v>
       </c>
       <c r="AQ11" t="n">
-        <v>64.3019</v>
+        <v>64.3013</v>
       </c>
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="n">
         <v>85</v>
       </c>
       <c r="AT11" t="n">
-        <v>61.9</v>
+        <v>61.4</v>
       </c>
       <c r="AU11" t="n">
         <v>78.09999999999999</v>
@@ -2899,10 +2899,10 @@
         <v>67.81999999999999</v>
       </c>
       <c r="AZ11" t="n">
-        <v>1.05</v>
+        <v>0.86</v>
       </c>
       <c r="BA11" t="n">
-        <v>4.97</v>
+        <v>4.77</v>
       </c>
       <c r="BB11" t="inlineStr"/>
       <c r="BC11" t="inlineStr"/>
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>VWCE.DE: scenario base Accumulate Carefully, score 72.6, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.1%.</t>
+          <t>VWCE.DE: scenario base Accumulate Carefully, score 72.6, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.0%.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -3026,10 +3026,10 @@
         </is>
       </c>
       <c r="Y12" t="n">
-        <v>1.01</v>
+        <v>0.96</v>
       </c>
       <c r="Z12" t="n">
-        <v>20.25</v>
+        <v>20.19</v>
       </c>
       <c r="AA12" t="n">
         <v>13</v>
@@ -3050,13 +3050,13 @@
         </is>
       </c>
       <c r="AG12" t="n">
-        <v>166.3</v>
+        <v>166.22</v>
       </c>
       <c r="AH12" t="n">
         <v>71.90000000000001</v>
       </c>
       <c r="AI12" t="n">
-        <v>64</v>
+        <v>63.9</v>
       </c>
       <c r="AJ12" t="n">
         <v>67.5</v>
@@ -3065,29 +3065,29 @@
         <v>82.8</v>
       </c>
       <c r="AL12" t="n">
-        <v>-1.53</v>
+        <v>-1.58</v>
       </c>
       <c r="AM12" t="n">
-        <v>12.52</v>
+        <v>12.46</v>
       </c>
       <c r="AN12" t="n">
-        <v>16.81</v>
+        <v>16.79</v>
       </c>
       <c r="AO12" t="n">
         <v>1.29</v>
       </c>
       <c r="AP12" t="n">
-        <v>166.1828</v>
+        <v>166.1812</v>
       </c>
       <c r="AQ12" t="n">
-        <v>155.4232</v>
+        <v>155.4228</v>
       </c>
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="n">
         <v>85</v>
       </c>
       <c r="AT12" t="n">
-        <v>64</v>
+        <v>63.9</v>
       </c>
       <c r="AU12" t="n">
         <v>67.5</v>
@@ -3105,10 +3105,10 @@
         <v>168.54</v>
       </c>
       <c r="AZ12" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.02</v>
       </c>
       <c r="BA12" t="n">
-        <v>7</v>
+        <v>6.95</v>
       </c>
       <c r="BB12" t="inlineStr"/>
       <c r="BC12" t="inlineStr"/>
@@ -3144,10 +3144,10 @@
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>71.7</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="F13" t="n">
-        <v>72.5</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -3161,7 +3161,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>score 71.7; priority 72.5; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 71.6; priority 72.4; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -3181,7 +3181,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>SXR8.DE: scenario base Accumulate Carefully, score 71.7, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.1%.</t>
+          <t>SXR8.DE: scenario base Accumulate Carefully, score 71.6, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.0%.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -3232,10 +3232,10 @@
         </is>
       </c>
       <c r="Y13" t="n">
-        <v>2.08</v>
+        <v>1.95</v>
       </c>
       <c r="Z13" t="n">
-        <v>18.86</v>
+        <v>18.71</v>
       </c>
       <c r="AA13" t="n">
         <v>14.25</v>
@@ -3256,13 +3256,13 @@
         </is>
       </c>
       <c r="AG13" t="n">
-        <v>712.52</v>
+        <v>711.62</v>
       </c>
       <c r="AH13" t="n">
-        <v>69.09999999999999</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="AI13" t="n">
-        <v>65.90000000000001</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="AJ13" t="n">
         <v>64.2</v>
@@ -3271,29 +3271,29 @@
         <v>82.8</v>
       </c>
       <c r="AL13" t="n">
-        <v>-1.61</v>
+        <v>-1.73</v>
       </c>
       <c r="AM13" t="n">
-        <v>13.79</v>
+        <v>13.64</v>
       </c>
       <c r="AN13" t="n">
-        <v>17.32</v>
+        <v>17.27</v>
       </c>
       <c r="AO13" t="n">
-        <v>1.22</v>
+        <v>1.21</v>
       </c>
       <c r="AP13" t="n">
-        <v>711.6136</v>
+        <v>711.5956</v>
       </c>
       <c r="AQ13" t="n">
-        <v>663.8201</v>
+        <v>663.8156</v>
       </c>
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="n">
         <v>85</v>
       </c>
       <c r="AT13" t="n">
-        <v>65.90000000000001</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="AU13" t="n">
         <v>64.2</v>
@@ -3311,10 +3311,10 @@
         <v>721.0599999999999</v>
       </c>
       <c r="AZ13" t="n">
-        <v>0.13</v>
+        <v>0</v>
       </c>
       <c r="BA13" t="n">
-        <v>7.34</v>
+        <v>7.2</v>
       </c>
       <c r="BB13" t="inlineStr"/>
       <c r="BC13" t="inlineStr"/>
@@ -3350,10 +3350,10 @@
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>69.09999999999999</v>
+        <v>69</v>
       </c>
       <c r="F14" t="n">
-        <v>70.8</v>
+        <v>70.7</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -3367,7 +3367,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>score 69.1; priority 70.8; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 69.0; priority 70.7; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>SWDA.MI: scenario base Accumulate Carefully, score 69.1, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.1%.</t>
+          <t>SWDA.MI: scenario base Accumulate Carefully, score 69.0, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.1%.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -3438,10 +3438,10 @@
         </is>
       </c>
       <c r="Y14" t="n">
-        <v>1.88</v>
+        <v>1.82</v>
       </c>
       <c r="Z14" t="n">
-        <v>18.82</v>
+        <v>18.75</v>
       </c>
       <c r="AA14" t="n">
         <v>13.2</v>
@@ -3462,50 +3462,50 @@
         </is>
       </c>
       <c r="AG14" t="n">
-        <v>126.51</v>
+        <v>126.43</v>
       </c>
       <c r="AH14" t="n">
         <v>71</v>
       </c>
       <c r="AI14" t="n">
-        <v>64.90000000000001</v>
+        <v>64.7</v>
       </c>
       <c r="AJ14" t="n">
         <v>66.90000000000001</v>
       </c>
       <c r="AK14" t="n">
-        <v>79.7</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="AL14" t="n">
-        <v>-1.82</v>
+        <v>-1.89</v>
       </c>
       <c r="AM14" t="n">
-        <v>12.54</v>
+        <v>12.47</v>
       </c>
       <c r="AN14" t="n">
-        <v>16.65</v>
+        <v>16.62</v>
       </c>
       <c r="AO14" t="n">
         <v>1.26</v>
       </c>
       <c r="AP14" t="n">
-        <v>126.583</v>
+        <v>126.5814</v>
       </c>
       <c r="AQ14" t="n">
-        <v>118.3545</v>
+        <v>118.3541</v>
       </c>
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="n">
         <v>65</v>
       </c>
       <c r="AT14" t="n">
-        <v>64.90000000000001</v>
+        <v>64.7</v>
       </c>
       <c r="AU14" t="n">
         <v>66.90000000000001</v>
       </c>
       <c r="AV14" t="n">
-        <v>79.7</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="AW14" t="n">
         <v>757</v>
@@ -3517,10 +3517,10 @@
         <v>128.21</v>
       </c>
       <c r="AZ14" t="n">
-        <v>-0.06</v>
+        <v>-0.12</v>
       </c>
       <c r="BA14" t="n">
-        <v>6.89</v>
+        <v>6.82</v>
       </c>
       <c r="BB14" t="inlineStr"/>
       <c r="BC14" t="inlineStr"/>
@@ -3593,7 +3593,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>EIMI.MI: scenario base Accumulate Carefully, score 69.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.4%.</t>
+          <t>EIMI.MI: scenario base Accumulate Carefully, score 69.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.5%.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -3644,10 +3644,10 @@
         </is>
       </c>
       <c r="Y15" t="n">
-        <v>-4.5</v>
+        <v>-4.47</v>
       </c>
       <c r="Z15" t="n">
-        <v>29.66</v>
+        <v>29.71</v>
       </c>
       <c r="AA15" t="n">
         <v>17.13</v>
@@ -3668,13 +3668,13 @@
         </is>
       </c>
       <c r="AG15" t="n">
-        <v>47.01</v>
+        <v>47.025</v>
       </c>
       <c r="AH15" t="n">
         <v>66.7</v>
       </c>
       <c r="AI15" t="n">
-        <v>58.9</v>
+        <v>59</v>
       </c>
       <c r="AJ15" t="n">
         <v>64.09999999999999</v>
@@ -3683,29 +3683,29 @@
         <v>82.8</v>
       </c>
       <c r="AL15" t="n">
-        <v>-0.28</v>
+        <v>-0.24</v>
       </c>
       <c r="AM15" t="n">
-        <v>12.96</v>
+        <v>13</v>
       </c>
       <c r="AN15" t="n">
-        <v>18.13</v>
+        <v>18.14</v>
       </c>
       <c r="AO15" t="n">
         <v>1.06</v>
       </c>
       <c r="AP15" t="n">
-        <v>46.8154</v>
+        <v>46.8157</v>
       </c>
       <c r="AQ15" t="n">
-        <v>43.8669</v>
+        <v>43.867</v>
       </c>
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="n">
         <v>85</v>
       </c>
       <c r="AT15" t="n">
-        <v>58.9</v>
+        <v>59</v>
       </c>
       <c r="AU15" t="n">
         <v>64.09999999999999</v>
@@ -3723,10 +3723,10 @@
         <v>48.565</v>
       </c>
       <c r="AZ15" t="n">
-        <v>0.42</v>
+        <v>0.45</v>
       </c>
       <c r="BA15" t="n">
-        <v>7.17</v>
+        <v>7.2</v>
       </c>
       <c r="BB15" t="inlineStr"/>
       <c r="BC15" t="inlineStr"/>
@@ -3762,10 +3762,10 @@
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>68.3</v>
+        <v>68.2</v>
       </c>
       <c r="F16" t="n">
-        <v>69.7</v>
+        <v>69.5</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -3779,7 +3779,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>score 68.3; priority 69.7; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 68.2; priority 69.5; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -3799,7 +3799,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>EXSA.DE: scenario base Accumulate Carefully, score 68.3, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -1.7%.</t>
+          <t>EXSA.DE: scenario base Accumulate Carefully, score 68.2, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -1.9%.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -3850,10 +3850,10 @@
         </is>
       </c>
       <c r="Y16" t="n">
-        <v>0.06</v>
+        <v>-0.08</v>
       </c>
       <c r="Z16" t="n">
-        <v>17.85</v>
+        <v>17.68</v>
       </c>
       <c r="AA16" t="n">
         <v>12.77</v>
@@ -3874,50 +3874,50 @@
         </is>
       </c>
       <c r="AG16" t="n">
-        <v>63.67</v>
+        <v>63.58</v>
       </c>
       <c r="AH16" t="n">
         <v>71.2</v>
       </c>
       <c r="AI16" t="n">
-        <v>59.3</v>
+        <v>59</v>
       </c>
       <c r="AJ16" t="n">
         <v>71.59999999999999</v>
       </c>
       <c r="AK16" t="n">
-        <v>77.2</v>
+        <v>77</v>
       </c>
       <c r="AL16" t="n">
-        <v>-3.18</v>
+        <v>-3.32</v>
       </c>
       <c r="AM16" t="n">
-        <v>7.95</v>
+        <v>7.8</v>
       </c>
       <c r="AN16" t="n">
-        <v>14.46</v>
+        <v>14.41</v>
       </c>
       <c r="AO16" t="n">
         <v>1.13</v>
       </c>
       <c r="AP16" t="n">
-        <v>64.7812</v>
+        <v>64.7794</v>
       </c>
       <c r="AQ16" t="n">
-        <v>61.2112</v>
+        <v>61.2108</v>
       </c>
       <c r="AR16" t="inlineStr"/>
       <c r="AS16" t="n">
         <v>65</v>
       </c>
       <c r="AT16" t="n">
-        <v>59.3</v>
+        <v>59</v>
       </c>
       <c r="AU16" t="n">
         <v>71.59999999999999</v>
       </c>
       <c r="AV16" t="n">
-        <v>77.2</v>
+        <v>77</v>
       </c>
       <c r="AW16" t="n">
         <v>760</v>
@@ -3929,10 +3929,10 @@
         <v>65.68000000000001</v>
       </c>
       <c r="AZ16" t="n">
-        <v>-1.72</v>
+        <v>-1.85</v>
       </c>
       <c r="BA16" t="n">
-        <v>4.02</v>
+        <v>3.87</v>
       </c>
       <c r="BB16" t="inlineStr"/>
       <c r="BC16" t="inlineStr"/>
@@ -3968,10 +3968,10 @@
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>66.90000000000001</v>
+        <v>66.8</v>
       </c>
       <c r="F17" t="n">
-        <v>69.40000000000001</v>
+        <v>69.3</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -3985,7 +3985,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>score 66.9; priority 69.4; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 66.8; priority 69.3; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -4005,7 +4005,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>IWQU.MI: scenario base Hold / Monitor, score 66.9, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.7%.</t>
+          <t>IWQU.MI: scenario base Hold / Monitor, score 66.8, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.9%.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -4056,10 +4056,10 @@
         </is>
       </c>
       <c r="Y17" t="n">
-        <v>1.38</v>
+        <v>1.23</v>
       </c>
       <c r="Z17" t="n">
-        <v>18.75</v>
+        <v>18.57</v>
       </c>
       <c r="AA17" t="n">
         <v>12.85</v>
@@ -4080,50 +4080,50 @@
         </is>
       </c>
       <c r="AG17" t="n">
-        <v>76.87</v>
+        <v>76.75</v>
       </c>
       <c r="AH17" t="n">
         <v>63.9</v>
       </c>
       <c r="AI17" t="n">
-        <v>63</v>
+        <v>62.6</v>
       </c>
       <c r="AJ17" t="n">
         <v>68.09999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>78.7</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="AL17" t="n">
-        <v>-2.18</v>
+        <v>-2.33</v>
       </c>
       <c r="AM17" t="n">
-        <v>10.64</v>
+        <v>10.46</v>
       </c>
       <c r="AN17" t="n">
-        <v>14.27</v>
+        <v>14.21</v>
       </c>
       <c r="AO17" t="n">
         <v>1.11</v>
       </c>
       <c r="AP17" t="n">
-        <v>77.4234</v>
+        <v>77.42100000000001</v>
       </c>
       <c r="AQ17" t="n">
-        <v>72.5491</v>
+        <v>72.5485</v>
       </c>
       <c r="AR17" t="inlineStr"/>
       <c r="AS17" t="n">
         <v>65</v>
       </c>
       <c r="AT17" t="n">
-        <v>63</v>
+        <v>62.6</v>
       </c>
       <c r="AU17" t="n">
         <v>68.09999999999999</v>
       </c>
       <c r="AV17" t="n">
-        <v>78.7</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="AW17" t="n">
         <v>757</v>
@@ -4135,10 +4135,10 @@
         <v>78.37</v>
       </c>
       <c r="AZ17" t="n">
-        <v>-0.71</v>
+        <v>-0.87</v>
       </c>
       <c r="BA17" t="n">
-        <v>5.96</v>
+        <v>5.79</v>
       </c>
       <c r="BB17" t="inlineStr"/>
       <c r="BC17" t="inlineStr"/>
@@ -4178,10 +4178,10 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>72.5</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="F18" t="n">
-        <v>68.09999999999999</v>
+        <v>68.3</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>score 72.5; priority 68.1; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 72.6; priority 68.3; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -4215,7 +4215,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>GOOGL: scenario base Accumulate Carefully, score 72.5, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -0.2%.</t>
+          <t>GOOGL: scenario base Accumulate Carefully, score 72.6, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -0.1%.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -4262,10 +4262,10 @@
         </is>
       </c>
       <c r="Y18" t="n">
-        <v>-3.7</v>
+        <v>-3.59</v>
       </c>
       <c r="Z18" t="n">
-        <v>44.38</v>
+        <v>44.55</v>
       </c>
       <c r="AA18" t="n">
         <v>30.66</v>
@@ -4274,10 +4274,10 @@
         <v>-29.81</v>
       </c>
       <c r="AC18" t="n">
-        <v>17.36</v>
+        <v>17.38</v>
       </c>
       <c r="AD18" t="n">
-        <v>23.27</v>
+        <v>23.3</v>
       </c>
       <c r="AE18" t="inlineStr">
         <is>
@@ -4286,42 +4286,42 @@
       </c>
       <c r="AF18" t="inlineStr"/>
       <c r="AG18" t="n">
-        <v>346.1514</v>
+        <v>346.545</v>
       </c>
       <c r="AH18" t="inlineStr"/>
       <c r="AI18" t="inlineStr"/>
       <c r="AJ18" t="inlineStr"/>
       <c r="AK18" t="inlineStr"/>
       <c r="AL18" t="n">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="AM18" t="n">
-        <v>14.66</v>
+        <v>14.79</v>
       </c>
       <c r="AN18" t="n">
-        <v>36.49</v>
+        <v>36.54</v>
       </c>
       <c r="AO18" t="n">
         <v>1.19</v>
       </c>
       <c r="AP18" t="n">
-        <v>346.7072</v>
+        <v>346.7151</v>
       </c>
       <c r="AQ18" t="n">
-        <v>336.523</v>
+        <v>336.5249</v>
       </c>
       <c r="AR18" t="inlineStr"/>
       <c r="AS18" t="n">
         <v>65</v>
       </c>
       <c r="AT18" t="n">
-        <v>64.7</v>
+        <v>65</v>
       </c>
       <c r="AU18" t="n">
         <v>39.4</v>
       </c>
       <c r="AV18" t="n">
-        <v>79.5</v>
+        <v>79.7</v>
       </c>
       <c r="AW18" t="n">
         <v>752</v>
@@ -4333,10 +4333,10 @@
         <v>347.8364</v>
       </c>
       <c r="AZ18" t="n">
-        <v>-0.16</v>
+        <v>-0.05</v>
       </c>
       <c r="BA18" t="n">
-        <v>2.86</v>
+        <v>2.98</v>
       </c>
       <c r="BB18" t="inlineStr">
         <is>
@@ -4349,7 +4349,7 @@
         </is>
       </c>
       <c r="BD18" t="n">
-        <v>4233409069056</v>
+        <v>4237550157824</v>
       </c>
       <c r="BE18" t="n">
         <v>54.77</v>
@@ -4370,7 +4370,7 @@
         <v>100</v>
       </c>
       <c r="BK18" t="n">
-        <v>64.7</v>
+        <v>65</v>
       </c>
       <c r="BL18" t="n">
         <v>74.8</v>
@@ -4379,7 +4379,7 @@
         <v>39.4</v>
       </c>
       <c r="BN18" t="n">
-        <v>79.5</v>
+        <v>79.7</v>
       </c>
       <c r="BO18" t="inlineStr"/>
       <c r="BP18" t="inlineStr">
@@ -4410,10 +4410,10 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>70</v>
+        <v>70.3</v>
       </c>
       <c r="F19" t="n">
-        <v>67.59999999999999</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -4427,7 +4427,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>score 70.0; priority 67.6; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 70.3; priority 68.1; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>AMZN: scenario base Accumulate Carefully, score 70.0, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -1.0%.</t>
+          <t>AMZN: scenario base Accumulate Carefully, score 70.3, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -0.6%.</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -4494,22 +4494,22 @@
         </is>
       </c>
       <c r="Y19" t="n">
-        <v>6.01</v>
+        <v>6.47</v>
       </c>
       <c r="Z19" t="n">
-        <v>9.970000000000001</v>
+        <v>10.45</v>
       </c>
       <c r="AA19" t="n">
-        <v>32.33</v>
+        <v>32.32</v>
       </c>
       <c r="AB19" t="n">
         <v>-30.88</v>
       </c>
       <c r="AC19" t="n">
-        <v>20.34</v>
+        <v>20.43</v>
       </c>
       <c r="AD19" t="n">
-        <v>24.3</v>
+        <v>24.41</v>
       </c>
       <c r="AE19" t="inlineStr">
         <is>
@@ -4518,42 +4518,42 @@
       </c>
       <c r="AF19" t="inlineStr"/>
       <c r="AG19" t="n">
-        <v>252.88</v>
+        <v>253.99</v>
       </c>
       <c r="AH19" t="inlineStr"/>
       <c r="AI19" t="inlineStr"/>
       <c r="AJ19" t="inlineStr"/>
       <c r="AK19" t="inlineStr"/>
       <c r="AL19" t="n">
-        <v>-4.62</v>
+        <v>-4.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>21.77</v>
+        <v>22.3</v>
       </c>
       <c r="AN19" t="n">
-        <v>20.57</v>
+        <v>20.74</v>
       </c>
       <c r="AO19" t="n">
         <v>0.64</v>
       </c>
       <c r="AP19" t="n">
-        <v>255.457</v>
+        <v>255.4792</v>
       </c>
       <c r="AQ19" t="n">
-        <v>239.9307</v>
+        <v>239.9362</v>
       </c>
       <c r="AR19" t="inlineStr"/>
       <c r="AS19" t="n">
         <v>65</v>
       </c>
       <c r="AT19" t="n">
-        <v>74</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="AU19" t="n">
         <v>36.5</v>
       </c>
       <c r="AV19" t="n">
-        <v>78.2</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="AW19" t="n">
         <v>752</v>
@@ -4565,10 +4565,10 @@
         <v>266.43</v>
       </c>
       <c r="AZ19" t="n">
-        <v>-1.02</v>
+        <v>-0.58</v>
       </c>
       <c r="BA19" t="n">
-        <v>5.39</v>
+        <v>5.86</v>
       </c>
       <c r="BB19" t="inlineStr">
         <is>
@@ -4581,7 +4581,7 @@
         </is>
       </c>
       <c r="BD19" t="n">
-        <v>2727464927232</v>
+        <v>2739615825920</v>
       </c>
       <c r="BE19" t="n">
         <v>17.44</v>
@@ -4600,16 +4600,16 @@
         <v>86.40000000000001</v>
       </c>
       <c r="BK19" t="n">
-        <v>74</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="BL19" t="n">
-        <v>69.90000000000001</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="BM19" t="n">
         <v>36.5</v>
       </c>
       <c r="BN19" t="n">
-        <v>78.2</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="BO19" t="inlineStr"/>
       <c r="BP19" t="inlineStr">
@@ -4621,17 +4621,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4. Alert / monitoraggio</t>
+          <t>2. Rischio da controllare</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Microsoft Corporation</t>
+          <t>NVIDIA Corporation</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -4640,24 +4640,24 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>78.7</v>
+        <v>70.2</v>
       </c>
       <c r="F20" t="n">
-        <v>65.2</v>
+        <v>52.1</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>🟡 Metti alert / monitora</t>
+          <t>🟥 Solo size piccola</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 513.53. Trigger: prezzo 10.2% sopra MA50: evitare inseguimento.</t>
+          <t>Tieni in osservazione senza azione immediata; rivaluta dopo aggiornamento dati o news rilevanti.</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>score 78.7; priority 65.2; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 70.2; priority 52.1; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -4667,27 +4667,27 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Medium-high risk</t>
+          <t>High risk</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>prezzo 10.2% sopra MA50: evitare inseguimento</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>MSFT: scenario base Buy Watchlist, score 78.7, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 10.2%.</t>
+          <t>NVDA: scenario base Accumulate Carefully, score 70.2, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -0.3%.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 513.53 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 230.10 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 352.17 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+          <t>Scenario negativo: perdita area 189.80 o peggioramento trend; rischio attuale: High risk.</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -4697,23 +4697,23 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Buy Watchlist</t>
+          <t>Accumulate Carefully</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Constructive</t>
         </is>
       </c>
       <c r="S20" t="n">
-        <v>352.167</v>
+        <v>189.7976</v>
       </c>
       <c r="T20" t="n">
-        <v>513.53</v>
+        <v>230.1025</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>Microsoft Corporation</t>
+          <t>NVIDIA Corporation</t>
         </is>
       </c>
       <c r="V20" t="inlineStr"/>
@@ -4724,81 +4724,81 @@
         </is>
       </c>
       <c r="Y20" t="n">
-        <v>28.71</v>
+        <v>3.48</v>
       </c>
       <c r="Z20" t="n">
-        <v>1.01</v>
+        <v>20</v>
       </c>
       <c r="AA20" t="n">
-        <v>26.23</v>
+        <v>46.97</v>
       </c>
       <c r="AB20" t="n">
-        <v>-34.5</v>
+        <v>-36.88</v>
       </c>
       <c r="AC20" t="n">
-        <v>27.98</v>
+        <v>26.85</v>
       </c>
       <c r="AD20" t="n">
-        <v>21.29</v>
+        <v>13.58</v>
       </c>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>Titolo forte; resta necessario controllare prezzo, trimestrali e size.</t>
+          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
         </is>
       </c>
       <c r="AF20" t="inlineStr"/>
       <c r="AG20" t="n">
-        <v>501.96</v>
+        <v>212.09</v>
       </c>
       <c r="AH20" t="inlineStr"/>
       <c r="AI20" t="inlineStr"/>
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
       <c r="AL20" t="n">
-        <v>1.21</v>
+        <v>-5.76</v>
       </c>
       <c r="AM20" t="n">
-        <v>27.42</v>
+        <v>17.93</v>
       </c>
       <c r="AN20" t="n">
-        <v>14.98</v>
+        <v>67.56999999999999</v>
       </c>
       <c r="AO20" t="n">
-        <v>0.57</v>
+        <v>1.44</v>
       </c>
       <c r="AP20" t="n">
-        <v>455.3591</v>
+        <v>212.7057</v>
       </c>
       <c r="AQ20" t="n">
-        <v>429.8087</v>
+        <v>197.2551</v>
       </c>
       <c r="AR20" t="inlineStr"/>
       <c r="AS20" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="AT20" t="n">
-        <v>100</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="AU20" t="n">
-        <v>40.9</v>
+        <v>14.1</v>
       </c>
       <c r="AV20" t="n">
-        <v>57.8</v>
+        <v>79.3</v>
       </c>
       <c r="AW20" t="n">
         <v>752</v>
       </c>
       <c r="AX20" t="n">
-        <v>479.4474</v>
+        <v>208.247</v>
       </c>
       <c r="AY20" t="n">
-        <v>513.53</v>
+        <v>230.1025</v>
       </c>
       <c r="AZ20" t="n">
-        <v>10.23</v>
+        <v>-0.29</v>
       </c>
       <c r="BA20" t="n">
-        <v>16.79</v>
+        <v>7.52</v>
       </c>
       <c r="BB20" t="inlineStr">
         <is>
@@ -4807,46 +4807,46 @@
       </c>
       <c r="BC20" t="inlineStr">
         <is>
-          <t>Software - Infrastructure</t>
+          <t>Semiconductors</t>
         </is>
       </c>
       <c r="BD20" t="n">
-        <v>3727326969856</v>
+        <v>5121095761920</v>
       </c>
       <c r="BE20" t="n">
-        <v>40.3</v>
+        <v>63.66</v>
       </c>
       <c r="BF20" t="n">
-        <v>34.04</v>
+        <v>117.21</v>
       </c>
       <c r="BG20" t="n">
-        <v>17.7</v>
+        <v>105.9</v>
       </c>
       <c r="BH20" t="n">
-        <v>29.12</v>
+        <v>16.97</v>
       </c>
       <c r="BI20" t="n">
-        <v>73</v>
+        <v>46</v>
       </c>
       <c r="BJ20" t="n">
         <v>100</v>
       </c>
       <c r="BK20" t="n">
-        <v>100</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="BL20" t="n">
-        <v>65.3</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="BM20" t="n">
-        <v>40.9</v>
+        <v>14.1</v>
       </c>
       <c r="BN20" t="n">
-        <v>57.8</v>
+        <v>79.3</v>
       </c>
       <c r="BO20" t="inlineStr"/>
       <c r="BP20" t="inlineStr">
         <is>
-          <t>USA / Technology</t>
+          <t>USA / Semiconductors</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4875,7 @@
         <v>71.7</v>
       </c>
       <c r="F21" t="n">
-        <v>45.6</v>
+        <v>45.8</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -4889,7 +4889,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>score 71.7; priority 45.6; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 71.7; priority 45.8; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -4904,12 +4904,12 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>prezzo 9.8% sopra MA50: evitare inseguimento; vicino a resistenza 20D: attenzione a falso breakout</t>
+          <t>prezzo 9.7% sopra MA50: evitare inseguimento; vicino a resistenza 20D: attenzione a falso breakout</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>META: scenario base Accumulate Carefully, score 71.7, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 9.8%.</t>
+          <t>META: scenario base Accumulate Carefully, score 71.7, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 9.7%.</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -4956,10 +4956,10 @@
         </is>
       </c>
       <c r="Y21" t="n">
-        <v>16.73</v>
+        <v>16.67</v>
       </c>
       <c r="Z21" t="n">
-        <v>-11.65</v>
+        <v>-11.7</v>
       </c>
       <c r="AA21" t="n">
         <v>37.67</v>
@@ -4968,10 +4968,10 @@
         <v>-34.15</v>
       </c>
       <c r="AC21" t="n">
-        <v>24.89</v>
+        <v>24.87</v>
       </c>
       <c r="AD21" t="n">
-        <v>18.91</v>
+        <v>18.9</v>
       </c>
       <c r="AE21" t="inlineStr">
         <is>
@@ -4980,42 +4980,42 @@
       </c>
       <c r="AF21" t="inlineStr"/>
       <c r="AG21" t="n">
-        <v>661.25</v>
+        <v>660.87</v>
       </c>
       <c r="AH21" t="inlineStr"/>
       <c r="AI21" t="inlineStr"/>
       <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="inlineStr"/>
       <c r="AL21" t="n">
-        <v>11.14</v>
+        <v>11.08</v>
       </c>
       <c r="AM21" t="n">
-        <v>7.94</v>
+        <v>7.88</v>
       </c>
       <c r="AN21" t="n">
-        <v>29.04</v>
+        <v>29.01</v>
       </c>
       <c r="AO21" t="n">
         <v>0.77</v>
       </c>
       <c r="AP21" t="n">
-        <v>602.4692</v>
+        <v>602.4616</v>
       </c>
       <c r="AQ21" t="n">
-        <v>622.8271999999999</v>
+        <v>622.8253</v>
       </c>
       <c r="AR21" t="inlineStr"/>
       <c r="AS21" t="n">
         <v>85</v>
       </c>
       <c r="AT21" t="n">
-        <v>75.3</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="AU21" t="n">
         <v>27.5</v>
       </c>
       <c r="AV21" t="n">
-        <v>59.7</v>
+        <v>60</v>
       </c>
       <c r="AW21" t="n">
         <v>752</v>
@@ -5024,13 +5024,13 @@
         <v>543.67</v>
       </c>
       <c r="AY21" t="n">
-        <v>661.25</v>
+        <v>660.87</v>
       </c>
       <c r="AZ21" t="n">
-        <v>9.76</v>
+        <v>9.69</v>
       </c>
       <c r="BA21" t="n">
-        <v>6.17</v>
+        <v>6.11</v>
       </c>
       <c r="BB21" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         </is>
       </c>
       <c r="BD21" t="n">
-        <v>1684538523648</v>
+        <v>1683570425856</v>
       </c>
       <c r="BE21" t="n">
         <v>29.83</v>
@@ -5064,7 +5064,7 @@
         <v>100</v>
       </c>
       <c r="BK21" t="n">
-        <v>75.3</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="BL21" t="n">
         <v>72.3</v>
@@ -5073,7 +5073,7 @@
         <v>27.5</v>
       </c>
       <c r="BN21" t="n">
-        <v>59.7</v>
+        <v>60</v>
       </c>
       <c r="BO21" t="inlineStr"/>
       <c r="BP21" t="inlineStr">
@@ -5090,20 +5090,24 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SGLD.MI</t>
+          <t>STM.MI</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Invesco Physical Gold ETC</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
+          <t>STM.MI</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
       <c r="E22" t="n">
-        <v>55.9</v>
+        <v>38.5</v>
       </c>
       <c r="F22" t="n">
-        <v>59.4</v>
+        <v>32.3</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -5117,37 +5121,37 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>score 55.9; priority 59.4; trend: Weak; entry zone: Wait for trend repair; risk flag: Normal risk</t>
+          <t>score 38.5; priority 32.3; trend: No Data; entry zone: No Data; risk flag: No Data</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Wait for trend repair</t>
+          <t>No Data</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Normal risk</t>
+          <t>No Data</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma</t>
+          <t>Dati prezzo insufficienti.</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>SGLD.MI: scenario base Hold / Monitor, score 55.9, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -0.1%.</t>
+          <t>STM.MI: scenario base Avoid for Now, score 38.5, trend No Data. Entry zone: No Data. Distanza da MA50: n/d.</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 384.93 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area n/d con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 337.23 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area n/d o peggioramento trend; rischio attuale: No Data.</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -5157,136 +5161,106 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Hold / Monitor</t>
+          <t>Avoid for Now</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Weak</t>
-        </is>
-      </c>
-      <c r="S22" t="n">
-        <v>337.23</v>
-      </c>
-      <c r="T22" t="n">
-        <v>384.93</v>
-      </c>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>Invesco Physical Gold ETC</t>
-        </is>
-      </c>
-      <c r="W22" t="inlineStr">
-        <is>
-          <t>Defensive</t>
-        </is>
-      </c>
+          <t>No Data</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>STM.MI</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr">
         <is>
-          <t>Osservare</t>
-        </is>
-      </c>
-      <c r="Y22" t="n">
-        <v>-1.45</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>19.52</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>19</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>-22.72</v>
-      </c>
+          <t>Evitare per ora</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr"/>
       <c r="AC22" t="inlineStr"/>
       <c r="AD22" t="inlineStr"/>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>Strumento utile per bilanciare volatilità e rischio macro.</t>
-        </is>
-      </c>
-      <c r="AF22" t="inlineStr">
-        <is>
-          <t>Oro</t>
-        </is>
-      </c>
-      <c r="AG22" t="n">
-        <v>356.48</v>
-      </c>
-      <c r="AH22" t="n">
-        <v>66.09999999999999</v>
-      </c>
-      <c r="AI22" t="n">
-        <v>44.1</v>
-      </c>
-      <c r="AJ22" t="n">
-        <v>59</v>
-      </c>
-      <c r="AK22" t="n">
-        <v>75.09999999999999</v>
-      </c>
-      <c r="AL22" t="n">
-        <v>-2.18</v>
-      </c>
-      <c r="AM22" t="n">
-        <v>-14.62</v>
-      </c>
-      <c r="AN22" t="n">
-        <v>27.28</v>
-      </c>
-      <c r="AO22" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="AP22" t="n">
-        <v>356.7442</v>
-      </c>
-      <c r="AQ22" t="n">
-        <v>374.4401</v>
-      </c>
+          <t>Da monitorare con scenario positivo, base e negativo.</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr"/>
+      <c r="AG22" t="inlineStr"/>
+      <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr"/>
+      <c r="AJ22" t="inlineStr"/>
+      <c r="AK22" t="inlineStr"/>
+      <c r="AL22" t="inlineStr"/>
+      <c r="AM22" t="inlineStr"/>
+      <c r="AN22" t="inlineStr"/>
+      <c r="AO22" t="inlineStr"/>
+      <c r="AP22" t="inlineStr"/>
+      <c r="AQ22" t="inlineStr"/>
       <c r="AR22" t="inlineStr"/>
       <c r="AS22" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="AT22" t="n">
-        <v>44.1</v>
+        <v>0</v>
       </c>
       <c r="AU22" t="n">
-        <v>59</v>
+        <v>100</v>
       </c>
       <c r="AV22" t="n">
-        <v>75.09999999999999</v>
+        <v>0</v>
       </c>
       <c r="AW22" t="n">
-        <v>757</v>
-      </c>
-      <c r="AX22" t="n">
-        <v>356.48</v>
-      </c>
-      <c r="AY22" t="n">
-        <v>384.93</v>
-      </c>
-      <c r="AZ22" t="n">
-        <v>-0.07000000000000001</v>
-      </c>
-      <c r="BA22" t="n">
-        <v>-4.8</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AX22" t="inlineStr"/>
+      <c r="AY22" t="inlineStr"/>
+      <c r="AZ22" t="inlineStr"/>
+      <c r="BA22" t="inlineStr"/>
       <c r="BB22" t="inlineStr"/>
       <c r="BC22" t="inlineStr"/>
-      <c r="BD22" t="inlineStr"/>
+      <c r="BD22" t="n">
+        <v>0</v>
+      </c>
       <c r="BE22" t="inlineStr"/>
       <c r="BF22" t="inlineStr"/>
       <c r="BG22" t="inlineStr"/>
       <c r="BH22" t="inlineStr"/>
       <c r="BI22" t="inlineStr"/>
-      <c r="BJ22" t="inlineStr"/>
-      <c r="BK22" t="inlineStr"/>
-      <c r="BL22" t="inlineStr"/>
-      <c r="BM22" t="inlineStr"/>
-      <c r="BN22" t="inlineStr"/>
-      <c r="BO22" t="inlineStr"/>
-      <c r="BP22" t="inlineStr"/>
+      <c r="BJ22" t="n">
+        <v>50</v>
+      </c>
+      <c r="BK22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL22" t="n">
+        <v>50</v>
+      </c>
+      <c r="BM22" t="n">
+        <v>100</v>
+      </c>
+      <c r="BN22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO22" t="inlineStr">
+        <is>
+          <t>Nessun dato prezzo disponibile</t>
+        </is>
+      </c>
+      <c r="BP22" t="inlineStr">
+        <is>
+          <t>Italy / Semiconductors</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5296,24 +5270,20 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>STM.MI</t>
+          <t>EUNA.MI</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>STM.MI</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
+          <t>iShares Core Global Aggregate Bond</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
-        <v>38.5</v>
+        <v>28.6</v>
       </c>
       <c r="F23" t="n">
-        <v>32.3</v>
+        <v>27.9</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -5327,7 +5297,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>score 38.5; priority 32.3; trend: No Data; entry zone: No Data; risk flag: No Data</t>
+          <t>score 28.6; priority 27.9; trend: No Data; entry zone: No Data; risk flag: No Data</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -5347,7 +5317,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>STM.MI: scenario base Avoid for Now, score 38.5, trend No Data. Entry zone: No Data. Distanza da MA50: n/d.</t>
+          <t>EUNA.MI: scenario base Avoid for Now, score 28.6, trend No Data. Entry zone: No Data. Distanza da MA50: n/d.</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -5377,13 +5347,17 @@
       </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>STM.MI</t>
-        </is>
-      </c>
-      <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>iShares Core Global Aggregate Bond</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>Defensive</t>
+        </is>
+      </c>
       <c r="X23" t="inlineStr">
         <is>
           <t>Evitare per ora</t>
@@ -5397,22 +5371,38 @@
       <c r="AD23" t="inlineStr"/>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>Da monitorare con scenario positivo, base e negativo.</t>
-        </is>
-      </c>
-      <c r="AF23" t="inlineStr"/>
+          <t>Strumento utile per bilanciare volatilità e rischio macro.</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>Obbligazionario globale</t>
+        </is>
+      </c>
       <c r="AG23" t="inlineStr"/>
-      <c r="AH23" t="inlineStr"/>
-      <c r="AI23" t="inlineStr"/>
-      <c r="AJ23" t="inlineStr"/>
-      <c r="AK23" t="inlineStr"/>
+      <c r="AH23" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ23" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK23" t="n">
+        <v>0</v>
+      </c>
       <c r="AL23" t="inlineStr"/>
       <c r="AM23" t="inlineStr"/>
       <c r="AN23" t="inlineStr"/>
       <c r="AO23" t="inlineStr"/>
       <c r="AP23" t="inlineStr"/>
       <c r="AQ23" t="inlineStr"/>
-      <c r="AR23" t="inlineStr"/>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>Nessun dato prezzo disponibile</t>
+        </is>
+      </c>
       <c r="AS23" t="n">
         <v>0</v>
       </c>
@@ -5434,39 +5424,19 @@
       <c r="BA23" t="inlineStr"/>
       <c r="BB23" t="inlineStr"/>
       <c r="BC23" t="inlineStr"/>
-      <c r="BD23" t="n">
-        <v>0</v>
-      </c>
+      <c r="BD23" t="inlineStr"/>
       <c r="BE23" t="inlineStr"/>
       <c r="BF23" t="inlineStr"/>
       <c r="BG23" t="inlineStr"/>
       <c r="BH23" t="inlineStr"/>
       <c r="BI23" t="inlineStr"/>
-      <c r="BJ23" t="n">
-        <v>50</v>
-      </c>
-      <c r="BK23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL23" t="n">
-        <v>50</v>
-      </c>
-      <c r="BM23" t="n">
-        <v>100</v>
-      </c>
-      <c r="BN23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO23" t="inlineStr">
-        <is>
-          <t>Nessun dato prezzo disponibile</t>
-        </is>
-      </c>
-      <c r="BP23" t="inlineStr">
-        <is>
-          <t>Italy / Semiconductors</t>
-        </is>
-      </c>
+      <c r="BJ23" t="inlineStr"/>
+      <c r="BK23" t="inlineStr"/>
+      <c r="BL23" t="inlineStr"/>
+      <c r="BM23" t="inlineStr"/>
+      <c r="BN23" t="inlineStr"/>
+      <c r="BO23" t="inlineStr"/>
+      <c r="BP23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5476,64 +5446,64 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>EUNA.MI</t>
+          <t>SGLD.MI</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>iShares Core Global Aggregate Bond</t>
+          <t>Invesco Physical Gold ETC</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
-        <v>28.6</v>
+        <v>59.5</v>
       </c>
       <c r="F24" t="n">
-        <v>27.9</v>
+        <v>61.9</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>⚪ Evita per ora</t>
+          <t>⚪ Osserva</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Lascia fuori dalla lista operativa finché trend, score o rischio non migliorano.</t>
+          <t>Tieni in osservazione senza azione immediata; rivaluta dopo aggiornamento dati o news rilevanti.</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>score 28.6; priority 27.9; trend: No Data; entry zone: No Data; risk flag: No Data</t>
+          <t>score 59.5; priority 61.9; trend: Recovery; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>No Data</t>
+          <t>Constructive entry zone</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>No Data</t>
+          <t>Normal risk</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Dati prezzo insufficienti.</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>EUNA.MI: scenario base Avoid for Now, score 28.6, trend No Data. Entry zone: No Data. Distanza da MA50: n/d.</t>
+          <t>SGLD.MI: scenario base Hold / Monitor, score 59.5, trend Recovery. Entry zone: Constructive entry zone. Distanza da MA50: 0.3%.</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area n/d con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 384.93 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area n/d o peggioramento trend; rischio attuale: No Data.</t>
+          <t>Scenario negativo: perdita area 337.23 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -5543,20 +5513,24 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Avoid for Now</t>
+          <t>Hold / Monitor</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>No Data</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="S24" t="n">
+        <v>337.23</v>
+      </c>
+      <c r="T24" t="n">
+        <v>384.93</v>
+      </c>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>iShares Core Global Aggregate Bond</t>
+          <t>Invesco Physical Gold ETC</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
@@ -5566,13 +5540,21 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>Evitare per ora</t>
-        </is>
-      </c>
-      <c r="Y24" t="inlineStr"/>
-      <c r="Z24" t="inlineStr"/>
-      <c r="AA24" t="inlineStr"/>
-      <c r="AB24" t="inlineStr"/>
+          <t>Osservare</t>
+        </is>
+      </c>
+      <c r="Y24" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>19.97</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>18.99</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>-22.72</v>
+      </c>
       <c r="AC24" t="inlineStr"/>
       <c r="AD24" t="inlineStr"/>
       <c r="AE24" t="inlineStr">
@@ -5582,52 +5564,70 @@
       </c>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>Obbligazionario globale</t>
-        </is>
-      </c>
-      <c r="AG24" t="inlineStr"/>
+          <t>Oro</t>
+        </is>
+      </c>
+      <c r="AG24" t="n">
+        <v>357.81</v>
+      </c>
       <c r="AH24" t="n">
-        <v>34.2</v>
+        <v>66.2</v>
       </c>
       <c r="AI24" t="n">
-        <v>0</v>
+        <v>44.9</v>
       </c>
       <c r="AJ24" t="n">
-        <v>100</v>
+        <v>59</v>
       </c>
       <c r="AK24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL24" t="inlineStr"/>
-      <c r="AM24" t="inlineStr"/>
-      <c r="AN24" t="inlineStr"/>
-      <c r="AO24" t="inlineStr"/>
-      <c r="AP24" t="inlineStr"/>
-      <c r="AQ24" t="inlineStr"/>
-      <c r="AR24" t="inlineStr">
-        <is>
-          <t>Nessun dato prezzo disponibile</t>
-        </is>
-      </c>
+        <v>78.2</v>
+      </c>
+      <c r="AL24" t="n">
+        <v>-1.82</v>
+      </c>
+      <c r="AM24" t="n">
+        <v>-14.3</v>
+      </c>
+      <c r="AN24" t="n">
+        <v>27.44</v>
+      </c>
+      <c r="AO24" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="AP24" t="n">
+        <v>356.7708</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>374.4467</v>
+      </c>
+      <c r="AR24" t="inlineStr"/>
       <c r="AS24" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="AT24" t="n">
-        <v>0</v>
+        <v>44.9</v>
       </c>
       <c r="AU24" t="n">
-        <v>100</v>
+        <v>59</v>
       </c>
       <c r="AV24" t="n">
-        <v>0</v>
+        <v>78.2</v>
       </c>
       <c r="AW24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX24" t="inlineStr"/>
-      <c r="AY24" t="inlineStr"/>
-      <c r="AZ24" t="inlineStr"/>
-      <c r="BA24" t="inlineStr"/>
+        <v>757</v>
+      </c>
+      <c r="AX24" t="n">
+        <v>357.81</v>
+      </c>
+      <c r="AY24" t="n">
+        <v>384.93</v>
+      </c>
+      <c r="AZ24" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="BA24" t="n">
+        <v>-4.44</v>
+      </c>
       <c r="BB24" t="inlineStr"/>
       <c r="BC24" t="inlineStr"/>
       <c r="BD24" t="inlineStr"/>

</xml_diff>

<commit_message>
Apply AlphaForge patch: alpha_forge_v12_fineco_real_patch.zip
</commit_message>
<xml_diff>
--- a/AlphaForge_Action_Plan.xlsx
+++ b/AlphaForge_Action_Plan.xlsx
@@ -776,10 +776,10 @@
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>67</v>
+        <v>66.7</v>
       </c>
       <c r="F2" t="n">
-        <v>69.59999999999999</v>
+        <v>69.3</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>score 67.0; priority 69.6; trend: Bullish; entry zone: Constructive entry zone; risk flag: Medium-high risk</t>
+          <t>score 66.7; priority 69.3; trend: Bullish; entry zone: Constructive entry zone; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>RBOT.MI: scenario base Hold / Monitor, score 67.0, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.7%.</t>
+          <t>RBOT.MI: scenario base Hold / Monitor, score 66.7, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.4%.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="Y2" t="n">
-        <v>7.38</v>
+        <v>7.07</v>
       </c>
       <c r="Z2" t="n">
-        <v>30.82</v>
+        <v>30.44</v>
       </c>
       <c r="AA2" t="n">
-        <v>22.7</v>
+        <v>22.71</v>
       </c>
       <c r="AB2" t="n">
         <v>-29.37</v>
@@ -888,13 +888,13 @@
         </is>
       </c>
       <c r="AG2" t="n">
-        <v>19.236</v>
+        <v>19.18</v>
       </c>
       <c r="AH2" t="n">
-        <v>56.1</v>
+        <v>55.9</v>
       </c>
       <c r="AI2" t="n">
-        <v>75.7</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="AJ2" t="n">
         <v>44.3</v>
@@ -903,29 +903,29 @@
         <v>82.8</v>
       </c>
       <c r="AL2" t="n">
-        <v>-0.42</v>
+        <v>-0.71</v>
       </c>
       <c r="AM2" t="n">
-        <v>12.69</v>
+        <v>12.36</v>
       </c>
       <c r="AN2" t="n">
-        <v>25.83</v>
+        <v>25.71</v>
       </c>
       <c r="AO2" t="n">
-        <v>1.14</v>
+        <v>1.13</v>
       </c>
       <c r="AP2" t="n">
-        <v>18.9211</v>
+        <v>18.9199</v>
       </c>
       <c r="AQ2" t="n">
-        <v>16.8872</v>
+        <v>16.8869</v>
       </c>
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="n">
         <v>85</v>
       </c>
       <c r="AT2" t="n">
-        <v>75.7</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="AU2" t="n">
         <v>49.3</v>
@@ -943,10 +943,10 @@
         <v>20.425</v>
       </c>
       <c r="AZ2" t="n">
-        <v>1.66</v>
+        <v>1.37</v>
       </c>
       <c r="BA2" t="n">
-        <v>13.91</v>
+        <v>13.58</v>
       </c>
       <c r="BB2" t="inlineStr"/>
       <c r="BC2" t="inlineStr"/>
@@ -986,10 +986,10 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>60.2</v>
+        <v>60.1</v>
       </c>
       <c r="F3" t="n">
-        <v>56.6</v>
+        <v>56.4</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>score 60.2; priority 56.6; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 60.1; priority 56.4; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>AMZN: scenario base Hold / Monitor, score 60.2, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -3.2%.</t>
+          <t>AMZN: scenario base Hold / Monitor, score 60.1, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -3.5%.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 245.96 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+          <t>Scenario negativo: perdita area 245.87 o peggioramento trend; rischio attuale: Medium-high risk.</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -1052,7 +1052,7 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>245.96</v>
+        <v>245.87</v>
       </c>
       <c r="T3" t="n">
         <v>278.09</v>
@@ -1070,22 +1070,22 @@
         </is>
       </c>
       <c r="Y3" t="n">
-        <v>-9.24</v>
+        <v>-9.470000000000001</v>
       </c>
       <c r="Z3" t="n">
-        <v>7.52</v>
+        <v>7.25</v>
       </c>
       <c r="AA3" t="n">
-        <v>31.84</v>
+        <v>31.85</v>
       </c>
       <c r="AB3" t="n">
         <v>-30.88</v>
       </c>
       <c r="AC3" t="n">
-        <v>19.83</v>
+        <v>19.78</v>
       </c>
       <c r="AD3" t="n">
-        <v>23.59</v>
+        <v>23.53</v>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
@@ -1094,57 +1094,57 @@
       </c>
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="n">
-        <v>246.48</v>
+        <v>245.87</v>
       </c>
       <c r="AH3" t="inlineStr"/>
       <c r="AI3" t="inlineStr"/>
       <c r="AJ3" t="inlineStr"/>
       <c r="AK3" t="inlineStr"/>
       <c r="AL3" t="n">
-        <v>-1.07</v>
+        <v>-1.32</v>
       </c>
       <c r="AM3" t="n">
-        <v>-7.01</v>
+        <v>-7.24</v>
       </c>
       <c r="AN3" t="n">
-        <v>23.02</v>
+        <v>22.92</v>
       </c>
       <c r="AO3" t="n">
         <v>0.72</v>
       </c>
       <c r="AP3" t="n">
-        <v>254.728</v>
+        <v>254.7158</v>
       </c>
       <c r="AQ3" t="n">
-        <v>243.3955</v>
+        <v>243.3925</v>
       </c>
       <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="n">
         <v>65</v>
       </c>
       <c r="AT3" t="n">
-        <v>34.7</v>
+        <v>34.2</v>
       </c>
       <c r="AU3" t="n">
         <v>37.1</v>
       </c>
       <c r="AV3" t="n">
-        <v>74.90000000000001</v>
+        <v>74.5</v>
       </c>
       <c r="AW3" t="n">
         <v>753</v>
       </c>
       <c r="AX3" t="n">
-        <v>246.5404</v>
+        <v>245.87</v>
       </c>
       <c r="AY3" t="n">
         <v>262.63</v>
       </c>
       <c r="AZ3" t="n">
-        <v>-3.21</v>
+        <v>-3.47</v>
       </c>
       <c r="BA3" t="n">
-        <v>1.29</v>
+        <v>1.02</v>
       </c>
       <c r="BB3" t="inlineStr">
         <is>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="BD3" t="n">
-        <v>2659262136320</v>
+        <v>2652030894080</v>
       </c>
       <c r="BE3" t="n">
         <v>17.44</v>
@@ -1176,16 +1176,16 @@
         <v>86.40000000000001</v>
       </c>
       <c r="BK3" t="n">
-        <v>34.7</v>
+        <v>34.2</v>
       </c>
       <c r="BL3" t="n">
-        <v>71.5</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="BM3" t="n">
         <v>37.1</v>
       </c>
       <c r="BN3" t="n">
-        <v>74.90000000000001</v>
+        <v>74.5</v>
       </c>
       <c r="BO3" t="inlineStr"/>
       <c r="BP3" t="inlineStr">
@@ -1216,10 +1216,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>67</v>
+        <v>68.5</v>
       </c>
       <c r="F4" t="n">
-        <v>52.9</v>
+        <v>54.5</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>score 67.0; priority 52.9; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 68.5; priority 54.5; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>ASML.AS: scenario base Hold / Monitor, score 67.0, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -0.0%.</t>
+          <t>ASML.AS: scenario base Accumulate Carefully, score 68.5, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 0.2%.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -1273,12 +1273,12 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Hold / Monitor</t>
+          <t>Accumulate Carefully</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Constructive</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="S4" t="n">
@@ -1300,10 +1300,10 @@
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>5.73</v>
+        <v>6</v>
       </c>
       <c r="Z4" t="n">
-        <v>62.78</v>
+        <v>63.19</v>
       </c>
       <c r="AA4" t="n">
         <v>39.88</v>
@@ -1312,10 +1312,10 @@
         <v>-44.77</v>
       </c>
       <c r="AC4" t="n">
-        <v>42.28</v>
+        <v>42.39</v>
       </c>
       <c r="AD4" t="n">
-        <v>26.8</v>
+        <v>26.87</v>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
@@ -1324,42 +1324,42 @@
       </c>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="n">
-        <v>1499</v>
+        <v>1502.8</v>
       </c>
       <c r="AH4" t="inlineStr"/>
       <c r="AI4" t="inlineStr"/>
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="inlineStr"/>
       <c r="AL4" t="n">
-        <v>-6</v>
+        <v>-5.76</v>
       </c>
       <c r="AM4" t="n">
-        <v>15.16</v>
+        <v>15.45</v>
       </c>
       <c r="AN4" t="n">
-        <v>40.12</v>
+        <v>40.24</v>
       </c>
       <c r="AO4" t="n">
         <v>1.01</v>
       </c>
       <c r="AP4" t="n">
-        <v>1499.3598</v>
+        <v>1499.4358</v>
       </c>
       <c r="AQ4" t="n">
-        <v>1385.9417</v>
+        <v>1385.9607</v>
       </c>
       <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="n">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="AT4" t="n">
-        <v>82.8</v>
+        <v>83.5</v>
       </c>
       <c r="AU4" t="n">
         <v>16.3</v>
       </c>
       <c r="AV4" t="n">
-        <v>79.7</v>
+        <v>82.8</v>
       </c>
       <c r="AW4" t="n">
         <v>766</v>
@@ -1371,10 +1371,10 @@
         <v>1653.9873</v>
       </c>
       <c r="AZ4" t="n">
-        <v>-0.02</v>
+        <v>0.22</v>
       </c>
       <c r="BA4" t="n">
-        <v>8.16</v>
+        <v>8.43</v>
       </c>
       <c r="BB4" t="inlineStr">
         <is>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="BD4" t="n">
-        <v>577741193216</v>
+        <v>579205791744</v>
       </c>
       <c r="BE4" t="n">
         <v>34.13</v>
@@ -1408,16 +1408,16 @@
         <v>100</v>
       </c>
       <c r="BK4" t="n">
-        <v>82.8</v>
+        <v>83.5</v>
       </c>
       <c r="BL4" t="n">
-        <v>40.8</v>
+        <v>40.6</v>
       </c>
       <c r="BM4" t="n">
         <v>16.3</v>
       </c>
       <c r="BN4" t="n">
-        <v>79.7</v>
+        <v>82.8</v>
       </c>
       <c r="BO4" t="inlineStr"/>
       <c r="BP4" t="inlineStr">
@@ -1448,10 +1448,10 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>68.40000000000001</v>
+        <v>68.3</v>
       </c>
       <c r="F5" t="n">
-        <v>49.3</v>
+        <v>49.1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1465,7 +1465,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>score 68.4; priority 49.3; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 68.3; priority 49.1; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>NVDA: scenario base Accumulate Carefully, score 68.4, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -3.7%.</t>
+          <t>NVDA: scenario base Accumulate Carefully, score 68.3, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -3.9%.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -1532,10 +1532,10 @@
         </is>
       </c>
       <c r="Y5" t="n">
-        <v>6.54</v>
+        <v>6.38</v>
       </c>
       <c r="Z5" t="n">
-        <v>6.53</v>
+        <v>6.36</v>
       </c>
       <c r="AA5" t="n">
         <v>46.63</v>
@@ -1544,10 +1544,10 @@
         <v>-36.88</v>
       </c>
       <c r="AC5" t="n">
-        <v>27.01</v>
+        <v>26.97</v>
       </c>
       <c r="AD5" t="n">
-        <v>13.42</v>
+        <v>13.4</v>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
@@ -1556,42 +1556,42 @@
       </c>
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="n">
-        <v>213.65</v>
+        <v>213.31</v>
       </c>
       <c r="AH5" t="inlineStr"/>
       <c r="AI5" t="inlineStr"/>
       <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="inlineStr"/>
       <c r="AL5" t="n">
-        <v>-6.45</v>
+        <v>-6.6</v>
       </c>
       <c r="AM5" t="n">
-        <v>7.3</v>
+        <v>7.13</v>
       </c>
       <c r="AN5" t="n">
-        <v>73.7</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="AO5" t="n">
         <v>1.58</v>
       </c>
       <c r="AP5" t="n">
-        <v>221.9238</v>
+        <v>221.917</v>
       </c>
       <c r="AQ5" t="n">
-        <v>203.9825</v>
+        <v>203.9808</v>
       </c>
       <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="n">
         <v>65</v>
       </c>
       <c r="AT5" t="n">
-        <v>65.2</v>
+        <v>64.8</v>
       </c>
       <c r="AU5" t="n">
         <v>14.5</v>
       </c>
       <c r="AV5" t="n">
-        <v>74.2</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="AW5" t="n">
         <v>753</v>
@@ -1603,10 +1603,10 @@
         <v>239.24</v>
       </c>
       <c r="AZ5" t="n">
-        <v>-3.73</v>
+        <v>-3.87</v>
       </c>
       <c r="BA5" t="n">
-        <v>4.73</v>
+        <v>4.58</v>
       </c>
       <c r="BB5" t="inlineStr">
         <is>
@@ -1619,7 +1619,7 @@
         </is>
       </c>
       <c r="BD5" t="n">
-        <v>5158764806144</v>
+        <v>5151158435840</v>
       </c>
       <c r="BE5" t="n">
         <v>63.66</v>
@@ -1640,7 +1640,7 @@
         <v>100</v>
       </c>
       <c r="BK5" t="n">
-        <v>65.2</v>
+        <v>64.8</v>
       </c>
       <c r="BL5" t="n">
         <v>77.7</v>
@@ -1649,7 +1649,7 @@
         <v>14.5</v>
       </c>
       <c r="BN5" t="n">
-        <v>74.2</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="BO5" t="inlineStr"/>
       <c r="BP5" t="inlineStr">
@@ -1666,20 +1666,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SMH</t>
+          <t>META</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>VanEck Semiconductor ETF</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
       <c r="E6" t="n">
-        <v>58.3</v>
+        <v>67.8</v>
       </c>
       <c r="F6" t="n">
-        <v>48.7</v>
+        <v>48.3</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1693,12 +1697,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>score 58.3; priority 48.7; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 67.8; priority 48.3; trend: Weak; entry zone: Wait for trend repair; risk flag: High risk</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Monitor / partial entry only</t>
+          <t>Wait for trend repair</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1708,22 +1712,22 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma</t>
+          <t>prezzo 6.8% sotto MA50: attendere recupero</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>SMH: scenario base Hold / Monitor, score 58.3, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -2.1%.</t>
+          <t>META: scenario base Hold / Monitor, score 67.8, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -6.8%.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 633.90 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 777.59 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 523.35 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 543.24 o peggioramento trend; rischio attuale: High risk.</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -1738,131 +1742,153 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Constructive</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="S6" t="n">
-        <v>523.35</v>
+        <v>543.2413</v>
       </c>
       <c r="T6" t="n">
-        <v>633.9</v>
-      </c>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>VanEck Semiconductor ETF</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>Thematic</t>
-        </is>
-      </c>
+        <v>777.59</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr">
         <is>
           <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y6" t="n">
-        <v>3.89</v>
+        <v>11.96</v>
       </c>
       <c r="Z6" t="n">
-        <v>55.13</v>
+        <v>-16.84</v>
       </c>
       <c r="AA6" t="n">
-        <v>37.36</v>
+        <v>38.53</v>
       </c>
       <c r="AB6" t="n">
-        <v>-35.74</v>
-      </c>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
+        <v>-34.15</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>21.25</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>17.5</v>
+      </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>Rischio elevato: usare solo come quota satellite e con size ridotta.</t>
-        </is>
-      </c>
-      <c r="AF6" t="inlineStr">
-        <is>
-          <t>Semiconduttori</t>
-        </is>
-      </c>
+          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="n">
-        <v>561.55</v>
-      </c>
-      <c r="AH6" t="n">
-        <v>55.3</v>
-      </c>
-      <c r="AI6" t="n">
-        <v>75.7</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>76.59999999999999</v>
-      </c>
+        <v>622.8150000000001</v>
+      </c>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
       <c r="AL6" t="n">
-        <v>-7.79</v>
+        <v>-14.12</v>
       </c>
       <c r="AM6" t="n">
-        <v>10.82</v>
+        <v>1.96</v>
       </c>
       <c r="AN6" t="n">
-        <v>60.69</v>
+        <v>27.72</v>
       </c>
       <c r="AO6" t="n">
-        <v>1.62</v>
+        <v>0.72</v>
       </c>
       <c r="AP6" t="n">
-        <v>573.4164</v>
+        <v>668.3628</v>
       </c>
       <c r="AQ6" t="n">
-        <v>518.8297</v>
+        <v>631.2616</v>
       </c>
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="n">
+        <v>35</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="AV6" t="n">
         <v>65</v>
-      </c>
-      <c r="AT6" t="n">
-        <v>75.7</v>
-      </c>
-      <c r="AU6" t="n">
-        <v>26.6</v>
-      </c>
-      <c r="AV6" t="n">
-        <v>76.59999999999999</v>
       </c>
       <c r="AW6" t="n">
         <v>753</v>
       </c>
       <c r="AX6" t="n">
-        <v>523.35</v>
+        <v>612.49</v>
       </c>
       <c r="AY6" t="n">
-        <v>633.9</v>
+        <v>762.5</v>
       </c>
       <c r="AZ6" t="n">
-        <v>-2.07</v>
+        <v>-6.82</v>
       </c>
       <c r="BA6" t="n">
-        <v>8.23</v>
-      </c>
-      <c r="BB6" t="inlineStr"/>
-      <c r="BC6" t="inlineStr"/>
-      <c r="BD6" t="inlineStr"/>
-      <c r="BE6" t="inlineStr"/>
-      <c r="BF6" t="inlineStr"/>
-      <c r="BG6" t="inlineStr"/>
-      <c r="BH6" t="inlineStr"/>
-      <c r="BI6" t="inlineStr"/>
-      <c r="BJ6" t="inlineStr"/>
-      <c r="BK6" t="inlineStr"/>
-      <c r="BL6" t="inlineStr"/>
-      <c r="BM6" t="inlineStr"/>
-      <c r="BN6" t="inlineStr"/>
+        <v>-1.35</v>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="BC6" t="inlineStr">
+        <is>
+          <t>Internet Content &amp; Information</t>
+        </is>
+      </c>
+      <c r="BD6" t="n">
+        <v>1592306171904</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>31.14</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>32.26</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>42.16</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>34</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>100</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>78.5</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="BN6" t="n">
+        <v>65</v>
+      </c>
       <c r="BO6" t="inlineStr"/>
-      <c r="BP6" t="inlineStr"/>
+      <c r="BP6" t="inlineStr">
+        <is>
+          <t>USA / Social &amp; AI</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1872,24 +1898,20 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>SMH</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Meta Platforms, Inc.</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
+          <t>VanEck Semiconductor ETF</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="F7" t="n">
-        <v>48.6</v>
+        <v>48.3</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1903,12 +1925,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>score 68.0; priority 48.6; trend: Weak; entry zone: Wait for trend repair; risk flag: High risk</t>
+          <t>score 58.0; priority 48.3; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Wait for trend repair</t>
+          <t>Monitor / partial entry only</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1918,22 +1940,22 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>prezzo 6.5% sotto MA50: attendere recupero</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>META: scenario base Accumulate Carefully, score 68.0, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -6.5%.</t>
+          <t>SMH: scenario base Hold / Monitor, score 58.0, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -2.4%.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 777.59 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 633.90 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 543.24 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 523.35 o peggioramento trend; rischio attuale: High risk.</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1943,158 +1965,136 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Accumulate Carefully</t>
+          <t>Hold / Monitor</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Constructive</t>
         </is>
       </c>
       <c r="S7" t="n">
-        <v>543.2413</v>
+        <v>523.35</v>
       </c>
       <c r="T7" t="n">
-        <v>777.59</v>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Meta Platforms, Inc.</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
+        <v>633.9</v>
+      </c>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>VanEck Semiconductor ETF</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Thematic</t>
+        </is>
+      </c>
       <c r="X7" t="inlineStr">
         <is>
           <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y7" t="n">
-        <v>12.32</v>
+        <v>3.52</v>
       </c>
       <c r="Z7" t="n">
-        <v>-16.57</v>
+        <v>54.58</v>
       </c>
       <c r="AA7" t="n">
-        <v>38.54</v>
+        <v>37.37</v>
       </c>
       <c r="AB7" t="n">
-        <v>-34.15</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>21.32</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>17.56</v>
-      </c>
+        <v>-35.74</v>
+      </c>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
-        </is>
-      </c>
-      <c r="AF7" t="inlineStr"/>
+          <t>Rischio elevato: usare solo come quota satellite e con size ridotta.</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>Semiconduttori</t>
+        </is>
+      </c>
       <c r="AG7" t="n">
-        <v>624.8</v>
-      </c>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
+        <v>559.5700000000001</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>74.8</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>76.09999999999999</v>
+      </c>
       <c r="AL7" t="n">
-        <v>-13.84</v>
+        <v>-8.119999999999999</v>
       </c>
       <c r="AM7" t="n">
-        <v>2.28</v>
+        <v>10.43</v>
       </c>
       <c r="AN7" t="n">
-        <v>27.86</v>
+        <v>60.5</v>
       </c>
       <c r="AO7" t="n">
-        <v>0.72</v>
+        <v>1.62</v>
       </c>
       <c r="AP7" t="n">
-        <v>668.4025</v>
+        <v>573.3768</v>
       </c>
       <c r="AQ7" t="n">
-        <v>631.2714999999999</v>
+        <v>518.8198</v>
       </c>
       <c r="AR7" t="inlineStr"/>
       <c r="AS7" t="n">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="AT7" t="n">
-        <v>64.5</v>
+        <v>74.8</v>
       </c>
       <c r="AU7" t="n">
-        <v>26.4</v>
+        <v>26.6</v>
       </c>
       <c r="AV7" t="n">
-        <v>65.5</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="AW7" t="n">
         <v>753</v>
       </c>
       <c r="AX7" t="n">
-        <v>612.49</v>
+        <v>523.35</v>
       </c>
       <c r="AY7" t="n">
-        <v>762.5</v>
+        <v>633.9</v>
       </c>
       <c r="AZ7" t="n">
-        <v>-6.52</v>
+        <v>-2.41</v>
       </c>
       <c r="BA7" t="n">
-        <v>-1.03</v>
-      </c>
-      <c r="BB7" t="inlineStr">
-        <is>
-          <t>Communication Services</t>
-        </is>
-      </c>
-      <c r="BC7" t="inlineStr">
-        <is>
-          <t>Internet Content &amp; Information</t>
-        </is>
-      </c>
-      <c r="BD7" t="n">
-        <v>1597509206016</v>
-      </c>
-      <c r="BE7" t="n">
-        <v>31.14</v>
-      </c>
-      <c r="BF7" t="n">
-        <v>32.26</v>
-      </c>
-      <c r="BG7" t="n">
-        <v>26.1</v>
-      </c>
-      <c r="BH7" t="n">
-        <v>42.16</v>
-      </c>
-      <c r="BI7" t="n">
-        <v>34</v>
-      </c>
-      <c r="BJ7" t="n">
-        <v>100</v>
-      </c>
-      <c r="BK7" t="n">
-        <v>64.5</v>
-      </c>
-      <c r="BL7" t="n">
-        <v>78.40000000000001</v>
-      </c>
-      <c r="BM7" t="n">
-        <v>26.4</v>
-      </c>
-      <c r="BN7" t="n">
-        <v>65.5</v>
-      </c>
+        <v>7.85</v>
+      </c>
+      <c r="BB7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr"/>
+      <c r="BD7" t="inlineStr"/>
+      <c r="BE7" t="inlineStr"/>
+      <c r="BF7" t="inlineStr"/>
+      <c r="BG7" t="inlineStr"/>
+      <c r="BH7" t="inlineStr"/>
+      <c r="BI7" t="inlineStr"/>
+      <c r="BJ7" t="inlineStr"/>
+      <c r="BK7" t="inlineStr"/>
+      <c r="BL7" t="inlineStr"/>
+      <c r="BM7" t="inlineStr"/>
+      <c r="BN7" t="inlineStr"/>
       <c r="BO7" t="inlineStr"/>
-      <c r="BP7" t="inlineStr">
-        <is>
-          <t>USA / Social &amp; AI</t>
-        </is>
-      </c>
+      <c r="BP7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2118,10 +2118,10 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>56</v>
+        <v>55.6</v>
       </c>
       <c r="F8" t="n">
-        <v>45.4</v>
+        <v>44.7</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -2135,7 +2135,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>score 56.0; priority 45.4; trend: Weak; entry zone: Wait for trend repair; risk flag: Medium-high risk</t>
+          <t>score 55.6; priority 44.7; trend: Weak; entry zone: Wait for trend repair; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -2150,12 +2150,12 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>prezzo 15.8% sotto MA50: attendere recupero; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo 16.4% sotto MA50: attendere recupero; vicino a supporto 60D: controllare tenuta e volumi</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>GOOGL: scenario base Hold / Monitor, score 56.0, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -15.8%.</t>
+          <t>GOOGL: scenario base Hold / Monitor, score 55.6, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -16.4%.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -2165,7 +2165,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 286.70 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+          <t>Scenario negativo: perdita area 284.28 o peggioramento trend; rischio attuale: Medium-high risk.</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -2184,7 +2184,7 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>286.6999</v>
+        <v>284.28</v>
       </c>
       <c r="T8" t="n">
         <v>357.5202</v>
@@ -2202,22 +2202,22 @@
         </is>
       </c>
       <c r="Y8" t="n">
-        <v>-19.45</v>
+        <v>-20.12</v>
       </c>
       <c r="Z8" t="n">
-        <v>7.46</v>
+        <v>6.56</v>
       </c>
       <c r="AA8" t="n">
-        <v>30.92</v>
+        <v>31.01</v>
       </c>
       <c r="AB8" t="n">
         <v>-29.81</v>
       </c>
       <c r="AC8" t="n">
-        <v>14.97</v>
+        <v>14.84</v>
       </c>
       <c r="AD8" t="n">
-        <v>18.73</v>
+        <v>18.57</v>
       </c>
       <c r="AE8" t="inlineStr">
         <is>
@@ -2226,57 +2226,57 @@
       </c>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="n">
-        <v>286.675</v>
+        <v>284.28</v>
       </c>
       <c r="AH8" t="inlineStr"/>
       <c r="AI8" t="inlineStr"/>
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr"/>
       <c r="AL8" t="n">
-        <v>-16.68</v>
+        <v>-17.38</v>
       </c>
       <c r="AM8" t="n">
-        <v>-25.41</v>
+        <v>-26.03</v>
       </c>
       <c r="AN8" t="n">
-        <v>32.63</v>
+        <v>32.26</v>
       </c>
       <c r="AO8" t="n">
-        <v>1.06</v>
+        <v>1.04</v>
       </c>
       <c r="AP8" t="n">
-        <v>340.2971</v>
+        <v>340.2492</v>
       </c>
       <c r="AQ8" t="n">
-        <v>340.6335</v>
+        <v>340.6215</v>
       </c>
       <c r="AR8" t="inlineStr"/>
       <c r="AS8" t="n">
         <v>35</v>
       </c>
       <c r="AT8" t="n">
-        <v>9.4</v>
+        <v>7.8</v>
       </c>
       <c r="AU8" t="n">
-        <v>39.1</v>
+        <v>38.9</v>
       </c>
       <c r="AV8" t="n">
-        <v>51.6</v>
+        <v>50.6</v>
       </c>
       <c r="AW8" t="n">
         <v>753</v>
       </c>
       <c r="AX8" t="n">
-        <v>286.6999</v>
+        <v>284.28</v>
       </c>
       <c r="AY8" t="n">
         <v>353.78</v>
       </c>
       <c r="AZ8" t="n">
-        <v>-15.75</v>
+        <v>-16.45</v>
       </c>
       <c r="BA8" t="n">
-        <v>-15.83</v>
+        <v>-16.54</v>
       </c>
       <c r="BB8" t="inlineStr">
         <is>
@@ -2289,7 +2289,7 @@
         </is>
       </c>
       <c r="BD8" t="n">
-        <v>3506933858304</v>
+        <v>3476725956608</v>
       </c>
       <c r="BE8" t="n">
         <v>54.77</v>
@@ -2310,16 +2310,16 @@
         <v>100</v>
       </c>
       <c r="BK8" t="n">
-        <v>9.4</v>
+        <v>7.8</v>
       </c>
       <c r="BL8" t="n">
-        <v>84.09999999999999</v>
+        <v>84.5</v>
       </c>
       <c r="BM8" t="n">
-        <v>39.1</v>
+        <v>38.9</v>
       </c>
       <c r="BN8" t="n">
-        <v>51.6</v>
+        <v>50.6</v>
       </c>
       <c r="BO8" t="inlineStr"/>
       <c r="BP8" t="inlineStr">
@@ -2346,10 +2346,10 @@
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>37.9</v>
+        <v>38.3</v>
       </c>
       <c r="F9" t="n">
-        <v>43.3</v>
+        <v>43.8</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -2363,7 +2363,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>score 37.9; priority 43.3; trend: Weak; entry zone: Wait for trend repair; risk flag: Medium-high risk</t>
+          <t>score 38.3; priority 43.8; trend: Weak; entry zone: Wait for trend repair; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -2378,12 +2378,12 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>prezzo 6.6% sotto MA50: attendere recupero; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo 6.2% sotto MA50: attendere recupero; vicino a supporto 60D: controllare tenuta e volumi</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>INRG.MI: scenario base Avoid for Now, score 37.9, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -6.6%.</t>
+          <t>INRG.MI: scenario base Avoid for Now, score 38.3, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -6.2%.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -2434,10 +2434,10 @@
         </is>
       </c>
       <c r="Y9" t="n">
-        <v>-10.55</v>
+        <v>-10.14</v>
       </c>
       <c r="Z9" t="n">
-        <v>-5.73</v>
+        <v>-5.3</v>
       </c>
       <c r="AA9" t="n">
         <v>24.07</v>
@@ -2458,50 +2458,50 @@
         </is>
       </c>
       <c r="AG9" t="n">
-        <v>8.071</v>
+        <v>8.108000000000001</v>
       </c>
       <c r="AH9" t="n">
-        <v>38.5</v>
+        <v>38.7</v>
       </c>
       <c r="AI9" t="n">
-        <v>20.7</v>
+        <v>21.6</v>
       </c>
       <c r="AJ9" t="n">
         <v>40.3</v>
       </c>
       <c r="AK9" t="n">
-        <v>65.40000000000001</v>
+        <v>66</v>
       </c>
       <c r="AL9" t="n">
-        <v>-6.54</v>
+        <v>-6.11</v>
       </c>
       <c r="AM9" t="n">
-        <v>-21.84</v>
+        <v>-21.48</v>
       </c>
       <c r="AN9" t="n">
-        <v>6.47</v>
+        <v>6.64</v>
       </c>
       <c r="AO9" t="n">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="AP9" t="n">
-        <v>8.6411</v>
+        <v>8.6418</v>
       </c>
       <c r="AQ9" t="n">
-        <v>9.3622</v>
+        <v>9.362399999999999</v>
       </c>
       <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="n">
         <v>35</v>
       </c>
       <c r="AT9" t="n">
-        <v>20.7</v>
+        <v>21.6</v>
       </c>
       <c r="AU9" t="n">
         <v>45.3</v>
       </c>
       <c r="AV9" t="n">
-        <v>65.40000000000001</v>
+        <v>66</v>
       </c>
       <c r="AW9" t="n">
         <v>758</v>
@@ -2513,10 +2513,10 @@
         <v>8.932</v>
       </c>
       <c r="AZ9" t="n">
-        <v>-6.6</v>
+        <v>-6.18</v>
       </c>
       <c r="BA9" t="n">
-        <v>-13.79</v>
+        <v>-13.4</v>
       </c>
       <c r="BB9" t="inlineStr"/>
       <c r="BC9" t="inlineStr"/>
@@ -2552,10 +2552,10 @@
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>56.5</v>
+        <v>56.9</v>
       </c>
       <c r="F10" t="n">
-        <v>37.4</v>
+        <v>39.3</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -2569,12 +2569,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>score 56.5; priority 37.4; trend: Bullish; entry zone: Extended - wait pullback; risk flag: High risk</t>
+          <t>score 56.9; priority 39.3; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Extended - wait pullback</t>
+          <t>Monitor / partial entry only</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -2584,12 +2584,12 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>prezzo 11.1% sopra MA50: evitare inseguimento</t>
+          <t>prezzo 10.5% sopra MA50: evitare inseguimento</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>WCLD.MI: scenario base Hold / Monitor, score 56.5, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 11.1%.</t>
+          <t>WCLD.MI: scenario base Hold / Monitor, score 56.9, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 10.5%.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -2640,13 +2640,13 @@
         </is>
       </c>
       <c r="Y10" t="n">
-        <v>28.83</v>
+        <v>28.09</v>
       </c>
       <c r="Z10" t="n">
-        <v>33.95</v>
+        <v>33.18</v>
       </c>
       <c r="AA10" t="n">
-        <v>35.24</v>
+        <v>35.25</v>
       </c>
       <c r="AB10" t="n">
         <v>-48.6</v>
@@ -2664,7 +2664,7 @@
         </is>
       </c>
       <c r="AG10" t="n">
-        <v>40.285</v>
+        <v>40.055</v>
       </c>
       <c r="AH10" t="n">
         <v>31.5</v>
@@ -2676,25 +2676,25 @@
         <v>13.8</v>
       </c>
       <c r="AK10" t="n">
-        <v>54.3</v>
+        <v>56.7</v>
       </c>
       <c r="AL10" t="n">
-        <v>13.54</v>
+        <v>12.89</v>
       </c>
       <c r="AM10" t="n">
-        <v>66.81</v>
+        <v>65.86</v>
       </c>
       <c r="AN10" t="n">
-        <v>17.04</v>
+        <v>16.82</v>
       </c>
       <c r="AO10" t="n">
         <v>0.48</v>
       </c>
       <c r="AP10" t="n">
-        <v>36.2532</v>
+        <v>36.2486</v>
       </c>
       <c r="AQ10" t="n">
-        <v>28.5749</v>
+        <v>28.5737</v>
       </c>
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="n">
@@ -2707,7 +2707,7 @@
         <v>18.8</v>
       </c>
       <c r="AV10" t="n">
-        <v>54.3</v>
+        <v>56.7</v>
       </c>
       <c r="AW10" t="n">
         <v>759</v>
@@ -2719,10 +2719,10 @@
         <v>41.05</v>
       </c>
       <c r="AZ10" t="n">
-        <v>11.12</v>
+        <v>10.5</v>
       </c>
       <c r="BA10" t="n">
-        <v>40.98</v>
+        <v>40.18</v>
       </c>
       <c r="BB10" t="inlineStr"/>
       <c r="BC10" t="inlineStr"/>
@@ -2765,7 +2765,7 @@
         <v>46.8</v>
       </c>
       <c r="F11" t="n">
-        <v>32.5</v>
+        <v>32.4</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -2779,7 +2779,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>score 46.8; priority 32.5; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 46.8; priority 32.4; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -2794,12 +2794,12 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>prezzo 9.9% sopra MA50: evitare inseguimento; vicino a resistenza 20D: attenzione a falso breakout</t>
+          <t>prezzo 10.0% sopra MA50: evitare inseguimento; vicino a resistenza 20D: attenzione a falso breakout</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>TSLA: scenario base High Risk, score 46.8, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 9.9%.</t>
+          <t>TSLA: scenario base High Risk, score 46.8, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 10.0%.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -2846,10 +2846,10 @@
         </is>
       </c>
       <c r="Y11" t="n">
-        <v>30.21</v>
+        <v>30.26</v>
       </c>
       <c r="Z11" t="n">
-        <v>-12.02</v>
+        <v>-11.98</v>
       </c>
       <c r="AA11" t="n">
         <v>57.81</v>
@@ -2858,10 +2858,10 @@
         <v>-53.77</v>
       </c>
       <c r="AC11" t="n">
-        <v>445.29</v>
+        <v>445.43</v>
       </c>
       <c r="AD11" t="n">
-        <v>188.01</v>
+        <v>188.07</v>
       </c>
       <c r="AE11" t="inlineStr">
         <is>
@@ -2870,42 +2870,42 @@
       </c>
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="n">
-        <v>405.2131</v>
+        <v>405.3752</v>
       </c>
       <c r="AH11" t="inlineStr"/>
       <c r="AI11" t="inlineStr"/>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
       <c r="AL11" t="n">
-        <v>14.21</v>
+        <v>14.25</v>
       </c>
       <c r="AM11" t="n">
-        <v>6.18</v>
+        <v>6.22</v>
       </c>
       <c r="AN11" t="n">
-        <v>27.22</v>
+        <v>27.24</v>
       </c>
       <c r="AO11" t="n">
         <v>0.47</v>
       </c>
       <c r="AP11" t="n">
-        <v>368.5473</v>
+        <v>368.5505</v>
       </c>
       <c r="AQ11" t="n">
-        <v>385.5051</v>
+        <v>385.5059</v>
       </c>
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="n">
         <v>85</v>
       </c>
       <c r="AT11" t="n">
-        <v>93</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="AU11" t="n">
         <v>0</v>
       </c>
       <c r="AV11" t="n">
-        <v>59</v>
+        <v>58.8</v>
       </c>
       <c r="AW11" t="n">
         <v>753</v>
@@ -2917,10 +2917,10 @@
         <v>407.46</v>
       </c>
       <c r="AZ11" t="n">
-        <v>9.949999999999999</v>
+        <v>9.98</v>
       </c>
       <c r="BA11" t="n">
-        <v>5.11</v>
+        <v>5.15</v>
       </c>
       <c r="BB11" t="inlineStr">
         <is>
@@ -2933,7 +2933,7 @@
         </is>
       </c>
       <c r="BD11" t="n">
-        <v>1601698004992</v>
+        <v>1602219409408</v>
       </c>
       <c r="BE11" t="n">
         <v>3.11</v>
@@ -2952,7 +2952,7 @@
         <v>53.7</v>
       </c>
       <c r="BK11" t="n">
-        <v>93</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="BL11" t="n">
         <v>0</v>
@@ -2961,7 +2961,7 @@
         <v>0</v>
       </c>
       <c r="BN11" t="n">
-        <v>59</v>
+        <v>58.8</v>
       </c>
       <c r="BO11" t="inlineStr"/>
       <c r="BP11" t="inlineStr">
@@ -3025,7 +3025,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>XDEV.MI: scenario base Buy Watchlist, score 78.8, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.6%.</t>
+          <t>XDEV.MI: scenario base Buy Watchlist, score 78.8, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.7%.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -3076,10 +3076,10 @@
         </is>
       </c>
       <c r="Y12" t="n">
-        <v>5.11</v>
+        <v>5.19</v>
       </c>
       <c r="Z12" t="n">
-        <v>47.38</v>
+        <v>47.5</v>
       </c>
       <c r="AA12" t="n">
         <v>14.1</v>
@@ -3100,13 +3100,13 @@
         </is>
       </c>
       <c r="AG12" t="n">
-        <v>74.09</v>
+        <v>74.15000000000001</v>
       </c>
       <c r="AH12" t="n">
-        <v>81.2</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="AI12" t="n">
-        <v>78.09999999999999</v>
+        <v>78.3</v>
       </c>
       <c r="AJ12" t="n">
         <v>68.8</v>
@@ -3115,29 +3115,29 @@
         <v>82.8</v>
       </c>
       <c r="AL12" t="n">
-        <v>-0.26</v>
+        <v>-0.18</v>
       </c>
       <c r="AM12" t="n">
-        <v>15.21</v>
+        <v>15.3</v>
       </c>
       <c r="AN12" t="n">
-        <v>28.68</v>
+        <v>28.71</v>
       </c>
       <c r="AO12" t="n">
-        <v>2.03</v>
+        <v>2.04</v>
       </c>
       <c r="AP12" t="n">
-        <v>73.619</v>
+        <v>73.6202</v>
       </c>
       <c r="AQ12" t="n">
-        <v>66.428</v>
+        <v>66.42829999999999</v>
       </c>
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="n">
         <v>85</v>
       </c>
       <c r="AT12" t="n">
-        <v>78.09999999999999</v>
+        <v>78.3</v>
       </c>
       <c r="AU12" t="n">
         <v>68.8</v>
@@ -3155,10 +3155,10 @@
         <v>74.98</v>
       </c>
       <c r="AZ12" t="n">
-        <v>0.64</v>
+        <v>0.72</v>
       </c>
       <c r="BA12" t="n">
-        <v>11.53</v>
+        <v>11.62</v>
       </c>
       <c r="BB12" t="inlineStr"/>
       <c r="BC12" t="inlineStr"/>
@@ -3194,10 +3194,10 @@
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>76.09999999999999</v>
+        <v>76</v>
       </c>
       <c r="F13" t="n">
-        <v>76.5</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -3206,12 +3206,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 71.66. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 71.47. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout.</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>score 76.1; priority 76.5; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 76.0; priority 76.6; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -3231,12 +3231,12 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>MVOL.MI: scenario base Accumulate Carefully, score 76.1, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 5.2%.</t>
+          <t>MVOL.MI: scenario base Accumulate Carefully, score 76.0, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 4.9%.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 71.66 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 71.47 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -3263,7 +3263,7 @@
         <v>66.25</v>
       </c>
       <c r="T13" t="n">
-        <v>71.66</v>
+        <v>71.47</v>
       </c>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
@@ -3282,10 +3282,10 @@
         </is>
       </c>
       <c r="Y13" t="n">
-        <v>7.69</v>
+        <v>7.38</v>
       </c>
       <c r="Z13" t="n">
-        <v>15.6</v>
+        <v>15.26</v>
       </c>
       <c r="AA13" t="n">
         <v>9.619999999999999</v>
@@ -3306,50 +3306,50 @@
         </is>
       </c>
       <c r="AG13" t="n">
-        <v>71.66</v>
+        <v>71.45</v>
       </c>
       <c r="AH13" t="n">
-        <v>70.5</v>
+        <v>70.3</v>
       </c>
       <c r="AI13" t="n">
-        <v>73.40000000000001</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="AJ13" t="n">
         <v>78.2</v>
       </c>
       <c r="AK13" t="n">
-        <v>78.09999999999999</v>
+        <v>79.3</v>
       </c>
       <c r="AL13" t="n">
-        <v>7.39</v>
+        <v>7.07</v>
       </c>
       <c r="AM13" t="n">
-        <v>14.49</v>
+        <v>14.16</v>
       </c>
       <c r="AN13" t="n">
-        <v>11.52</v>
+        <v>11.41</v>
       </c>
       <c r="AO13" t="n">
-        <v>1.2</v>
+        <v>1.19</v>
       </c>
       <c r="AP13" t="n">
-        <v>68.1456</v>
+        <v>68.1414</v>
       </c>
       <c r="AQ13" t="n">
-        <v>65.2871</v>
+        <v>65.2861</v>
       </c>
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="n">
         <v>85</v>
       </c>
       <c r="AT13" t="n">
-        <v>73.40000000000001</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="AU13" t="n">
         <v>78.2</v>
       </c>
       <c r="AV13" t="n">
-        <v>78.09999999999999</v>
+        <v>79.3</v>
       </c>
       <c r="AW13" t="n">
         <v>758</v>
@@ -3358,13 +3358,13 @@
         <v>67.20999999999999</v>
       </c>
       <c r="AY13" t="n">
-        <v>71.66</v>
+        <v>71.47</v>
       </c>
       <c r="AZ13" t="n">
-        <v>5.16</v>
+        <v>4.86</v>
       </c>
       <c r="BA13" t="n">
-        <v>9.76</v>
+        <v>9.44</v>
       </c>
       <c r="BB13" t="inlineStr"/>
       <c r="BC13" t="inlineStr"/>
@@ -3400,7 +3400,7 @@
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>73.8</v>
+        <v>73.7</v>
       </c>
       <c r="F14" t="n">
         <v>74.5</v>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>score 73.8; priority 74.5; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 73.7; priority 74.5; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>IWQU.MI: scenario base Accumulate Carefully, score 73.8, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.0%.</t>
+          <t>IWQU.MI: scenario base Accumulate Carefully, score 73.7, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 2.9%.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -3488,10 +3488,10 @@
         </is>
       </c>
       <c r="Y14" t="n">
-        <v>5.05</v>
+        <v>5.01</v>
       </c>
       <c r="Z14" t="n">
-        <v>19.7</v>
+        <v>19.65</v>
       </c>
       <c r="AA14" t="n">
         <v>12.65</v>
@@ -3512,13 +3512,13 @@
         </is>
       </c>
       <c r="AG14" t="n">
-        <v>81.18000000000001</v>
+        <v>81.15000000000001</v>
       </c>
       <c r="AH14" t="n">
-        <v>70.7</v>
+        <v>70.5</v>
       </c>
       <c r="AI14" t="n">
-        <v>69.09999999999999</v>
+        <v>69</v>
       </c>
       <c r="AJ14" t="n">
         <v>68.3</v>
@@ -3527,29 +3527,29 @@
         <v>82.8</v>
       </c>
       <c r="AL14" t="n">
-        <v>2.84</v>
+        <v>2.8</v>
       </c>
       <c r="AM14" t="n">
-        <v>11.85</v>
+        <v>11.81</v>
       </c>
       <c r="AN14" t="n">
-        <v>18.67</v>
+        <v>18.65</v>
       </c>
       <c r="AO14" t="n">
-        <v>1.48</v>
+        <v>1.47</v>
       </c>
       <c r="AP14" t="n">
-        <v>78.831</v>
+        <v>78.8304</v>
       </c>
       <c r="AQ14" t="n">
-        <v>74.3903</v>
+        <v>74.3901</v>
       </c>
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="n">
         <v>85</v>
       </c>
       <c r="AT14" t="n">
-        <v>69.09999999999999</v>
+        <v>69</v>
       </c>
       <c r="AU14" t="n">
         <v>68.3</v>
@@ -3567,10 +3567,10 @@
         <v>81.54000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>2.98</v>
+        <v>2.94</v>
       </c>
       <c r="BA14" t="n">
-        <v>9.130000000000001</v>
+        <v>9.09</v>
       </c>
       <c r="BB14" t="inlineStr"/>
       <c r="BC14" t="inlineStr"/>
@@ -3596,21 +3596,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>SWDA.MI</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Microsoft Corporation</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
+          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
-        <v>77.09999999999999</v>
+        <v>74.7</v>
       </c>
       <c r="F15" t="n">
         <v>74.40000000000001</v>
@@ -3622,42 +3618,42 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 543.45. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 132.27. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>score 77.1; priority 74.4; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 74.7; priority 74.4; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Monitor / partial entry only</t>
+          <t>Constructive entry zone</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Medium-high risk</t>
+          <t>Normal risk</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma</t>
+          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>MSFT: scenario base Accumulate Carefully, score 77.1, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 2.5%.</t>
+          <t>SWDA.MI: scenario base Accumulate Carefully, score 74.7, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 2.3%.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 543.45 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 132.27 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 479.45 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+          <t>Scenario negativo: perdita area 125.42 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -3676,149 +3672,127 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>479.4474</v>
+        <v>125.42</v>
       </c>
       <c r="T15" t="n">
-        <v>543.45</v>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>Microsoft Corporation</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
+        <v>132.27</v>
+      </c>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>Ridurre size / solo monitoraggio</t>
+          <t>Monitorare ingresso graduale</t>
         </is>
       </c>
       <c r="Y15" t="n">
-        <v>13.16</v>
+        <v>4.55</v>
       </c>
       <c r="Z15" t="n">
-        <v>-2.37</v>
+        <v>17.97</v>
       </c>
       <c r="AA15" t="n">
-        <v>26.12</v>
+        <v>13.08</v>
       </c>
       <c r="AB15" t="n">
-        <v>-34.5</v>
-      </c>
-      <c r="AC15" t="n">
-        <v>29.22</v>
-      </c>
-      <c r="AD15" t="n">
-        <v>22.14</v>
-      </c>
+        <v>-21.63</v>
+      </c>
+      <c r="AC15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr"/>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>Da monitorare con scenario positivo, base e negativo.</t>
-        </is>
-      </c>
-      <c r="AF15" t="inlineStr"/>
+          <t>Da monitorare: non è un segnale automatico di acquisto.</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>Azionario globale sviluppato</t>
+        </is>
+      </c>
       <c r="AG15" t="n">
-        <v>524.88</v>
-      </c>
-      <c r="AH15" t="inlineStr"/>
-      <c r="AI15" t="inlineStr"/>
-      <c r="AJ15" t="inlineStr"/>
-      <c r="AK15" t="inlineStr"/>
+        <v>131.85</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>67</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>67</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>82.8</v>
+      </c>
       <c r="AL15" t="n">
-        <v>2.34</v>
+        <v>2.1</v>
       </c>
       <c r="AM15" t="n">
-        <v>29.24</v>
+        <v>10.26</v>
       </c>
       <c r="AN15" t="n">
-        <v>16.85</v>
+        <v>21.18</v>
       </c>
       <c r="AO15" t="n">
-        <v>0.65</v>
+        <v>1.62</v>
       </c>
       <c r="AP15" t="n">
-        <v>511.9902</v>
+        <v>128.8848</v>
       </c>
       <c r="AQ15" t="n">
-        <v>436.5005</v>
+        <v>121.3353</v>
       </c>
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="n">
         <v>85</v>
       </c>
       <c r="AT15" t="n">
-        <v>85.40000000000001</v>
+        <v>67</v>
       </c>
       <c r="AU15" t="n">
-        <v>41.1</v>
+        <v>67</v>
       </c>
       <c r="AV15" t="n">
         <v>82.8</v>
       </c>
       <c r="AW15" t="n">
-        <v>753</v>
+        <v>758</v>
       </c>
       <c r="AX15" t="n">
-        <v>517.53</v>
+        <v>129.89</v>
       </c>
       <c r="AY15" t="n">
-        <v>543.45</v>
+        <v>132.27</v>
       </c>
       <c r="AZ15" t="n">
-        <v>2.46</v>
+        <v>2.3</v>
       </c>
       <c r="BA15" t="n">
-        <v>20.18</v>
-      </c>
-      <c r="BB15" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="BC15" t="inlineStr">
-        <is>
-          <t>Software - Infrastructure</t>
-        </is>
-      </c>
-      <c r="BD15" t="n">
-        <v>3895218667520</v>
-      </c>
-      <c r="BE15" t="n">
-        <v>40.3</v>
-      </c>
-      <c r="BF15" t="n">
-        <v>34.04</v>
-      </c>
-      <c r="BG15" t="n">
-        <v>17.7</v>
-      </c>
-      <c r="BH15" t="n">
-        <v>29.12</v>
-      </c>
-      <c r="BI15" t="n">
-        <v>74</v>
-      </c>
-      <c r="BJ15" t="n">
-        <v>100</v>
-      </c>
-      <c r="BK15" t="n">
-        <v>85.40000000000001</v>
-      </c>
-      <c r="BL15" t="n">
-        <v>62.6</v>
-      </c>
-      <c r="BM15" t="n">
-        <v>41.1</v>
-      </c>
-      <c r="BN15" t="n">
-        <v>82.8</v>
-      </c>
+        <v>8.67</v>
+      </c>
+      <c r="BB15" t="inlineStr"/>
+      <c r="BC15" t="inlineStr"/>
+      <c r="BD15" t="inlineStr"/>
+      <c r="BE15" t="inlineStr"/>
+      <c r="BF15" t="inlineStr"/>
+      <c r="BG15" t="inlineStr"/>
+      <c r="BH15" t="inlineStr"/>
+      <c r="BI15" t="inlineStr"/>
+      <c r="BJ15" t="inlineStr"/>
+      <c r="BK15" t="inlineStr"/>
+      <c r="BL15" t="inlineStr"/>
+      <c r="BM15" t="inlineStr"/>
+      <c r="BN15" t="inlineStr"/>
       <c r="BO15" t="inlineStr"/>
-      <c r="BP15" t="inlineStr">
-        <is>
-          <t>USA / Technology</t>
-        </is>
-      </c>
+      <c r="BP15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3828,20 +3802,20 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SWDA.MI</t>
+          <t>VWCE.DE</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
+          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>74.7</v>
+        <v>74.5</v>
       </c>
       <c r="F16" t="n">
-        <v>74.40000000000001</v>
+        <v>74.2</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -3850,12 +3824,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 132.27. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 173.56. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout; vicino a supporto 60D: controllare tenuta e volumi.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>score 74.7; priority 74.4; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 74.5; priority 74.2; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -3870,22 +3844,22 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout</t>
+          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout; vicino a supporto 60D: controllare tenuta e volumi</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>SWDA.MI: scenario base Accumulate Carefully, score 74.7, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 2.3%.</t>
+          <t>VWCE.DE: scenario base Accumulate Carefully, score 74.5, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.6%.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 132.27 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 173.56 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 125.42 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 165.26 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -3904,15 +3878,15 @@
         </is>
       </c>
       <c r="S16" t="n">
-        <v>125.42</v>
+        <v>165.26</v>
       </c>
       <c r="T16" t="n">
-        <v>132.27</v>
+        <v>173.56</v>
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
+          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
@@ -3926,16 +3900,16 @@
         </is>
       </c>
       <c r="Y16" t="n">
-        <v>4.58</v>
+        <v>4.11</v>
       </c>
       <c r="Z16" t="n">
-        <v>18</v>
+        <v>18.05</v>
       </c>
       <c r="AA16" t="n">
-        <v>13.08</v>
+        <v>12.93</v>
       </c>
       <c r="AB16" t="n">
-        <v>-21.63</v>
+        <v>-21.07</v>
       </c>
       <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="inlineStr"/>
@@ -3946,69 +3920,69 @@
       </c>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>Azionario globale sviluppato</t>
+          <t>Azionario globale</t>
         </is>
       </c>
       <c r="AG16" t="n">
-        <v>131.89</v>
+        <v>171.88</v>
       </c>
       <c r="AH16" t="n">
-        <v>77.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="AI16" t="n">
-        <v>67.09999999999999</v>
+        <v>65.5</v>
       </c>
       <c r="AJ16" t="n">
-        <v>67</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="AK16" t="n">
         <v>82.8</v>
       </c>
       <c r="AL16" t="n">
-        <v>2.13</v>
+        <v>1.24</v>
       </c>
       <c r="AM16" t="n">
-        <v>10.29</v>
+        <v>8.74</v>
       </c>
       <c r="AN16" t="n">
-        <v>21.19</v>
+        <v>20.96</v>
       </c>
       <c r="AO16" t="n">
         <v>1.62</v>
       </c>
       <c r="AP16" t="n">
-        <v>128.8856</v>
+        <v>169.2216</v>
       </c>
       <c r="AQ16" t="n">
-        <v>121.3355</v>
+        <v>159.5259</v>
       </c>
       <c r="AR16" t="inlineStr"/>
       <c r="AS16" t="n">
         <v>85</v>
       </c>
       <c r="AT16" t="n">
-        <v>67.09999999999999</v>
+        <v>65.5</v>
       </c>
       <c r="AU16" t="n">
-        <v>67</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="AV16" t="n">
         <v>82.8</v>
       </c>
       <c r="AW16" t="n">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="AX16" t="n">
-        <v>129.89</v>
+        <v>169.28</v>
       </c>
       <c r="AY16" t="n">
-        <v>132.27</v>
+        <v>173.56</v>
       </c>
       <c r="AZ16" t="n">
-        <v>2.33</v>
+        <v>1.57</v>
       </c>
       <c r="BA16" t="n">
-        <v>8.699999999999999</v>
+        <v>7.74</v>
       </c>
       <c r="BB16" t="inlineStr"/>
       <c r="BC16" t="inlineStr"/>
@@ -4034,20 +4008,20 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>VWCE.DE</t>
+          <t>SXR8.DE</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
+          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>74.59999999999999</v>
+        <v>74.2</v>
       </c>
       <c r="F17" t="n">
-        <v>74.2</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -4056,12 +4030,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 173.56. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout; vicino a supporto 60D: controllare tenuta e volumi.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 754.68. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>score 74.6; priority 74.2; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 74.2; priority 74.1; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -4076,22 +4050,22 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>VWCE.DE: scenario base Accumulate Carefully, score 74.6, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.6%.</t>
+          <t>SXR8.DE: scenario base Accumulate Carefully, score 74.2, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 2.6%.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 173.56 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 754.68 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 165.26 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 705.82 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -4110,15 +4084,15 @@
         </is>
       </c>
       <c r="S17" t="n">
-        <v>165.26</v>
+        <v>705.8200000000001</v>
       </c>
       <c r="T17" t="n">
-        <v>173.56</v>
+        <v>754.6799999999999</v>
       </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
+          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
@@ -4132,16 +4106,16 @@
         </is>
       </c>
       <c r="Y17" t="n">
-        <v>4.13</v>
+        <v>5.43</v>
       </c>
       <c r="Z17" t="n">
-        <v>18.08</v>
+        <v>18.09</v>
       </c>
       <c r="AA17" t="n">
-        <v>12.93</v>
+        <v>14.13</v>
       </c>
       <c r="AB17" t="n">
-        <v>-21.07</v>
+        <v>-23.32</v>
       </c>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="inlineStr"/>
@@ -4152,51 +4126,51 @@
       </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>Azionario globale</t>
+          <t>USA large cap</t>
         </is>
       </c>
       <c r="AG17" t="n">
-        <v>171.92</v>
+        <v>748.0599999999999</v>
       </c>
       <c r="AH17" t="n">
-        <v>77.90000000000001</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="AI17" t="n">
-        <v>65.59999999999999</v>
+        <v>69</v>
       </c>
       <c r="AJ17" t="n">
-        <v>67.59999999999999</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="AK17" t="n">
         <v>82.8</v>
       </c>
       <c r="AL17" t="n">
-        <v>1.26</v>
+        <v>2.09</v>
       </c>
       <c r="AM17" t="n">
-        <v>8.77</v>
+        <v>11.41</v>
       </c>
       <c r="AN17" t="n">
-        <v>20.97</v>
+        <v>22.14</v>
       </c>
       <c r="AO17" t="n">
-        <v>1.62</v>
+        <v>1.57</v>
       </c>
       <c r="AP17" t="n">
-        <v>169.2224</v>
+        <v>729.1328</v>
       </c>
       <c r="AQ17" t="n">
-        <v>159.5261</v>
+        <v>681.5774</v>
       </c>
       <c r="AR17" t="inlineStr"/>
       <c r="AS17" t="n">
         <v>85</v>
       </c>
       <c r="AT17" t="n">
-        <v>65.59999999999999</v>
+        <v>69</v>
       </c>
       <c r="AU17" t="n">
-        <v>67.59999999999999</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="AV17" t="n">
         <v>82.8</v>
@@ -4205,16 +4179,16 @@
         <v>760</v>
       </c>
       <c r="AX17" t="n">
-        <v>169.28</v>
+        <v>738.04</v>
       </c>
       <c r="AY17" t="n">
-        <v>173.56</v>
+        <v>754.6799999999999</v>
       </c>
       <c r="AZ17" t="n">
-        <v>1.59</v>
+        <v>2.6</v>
       </c>
       <c r="BA17" t="n">
-        <v>7.77</v>
+        <v>9.75</v>
       </c>
       <c r="BB17" t="inlineStr"/>
       <c r="BC17" t="inlineStr"/>
@@ -4240,20 +4214,24 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SXR8.DE</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
       <c r="E18" t="n">
-        <v>74.2</v>
+        <v>76.8</v>
       </c>
       <c r="F18" t="n">
-        <v>74.09999999999999</v>
+        <v>74</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -4262,42 +4240,42 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 754.68. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 543.45. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>score 74.2; priority 74.1; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 76.8; priority 74.0; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Constructive entry zone</t>
+          <t>Monitor / partial entry only</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Normal risk</t>
+          <t>Medium-high risk</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>SXR8.DE: scenario base Accumulate Carefully, score 74.2, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 2.6%.</t>
+          <t>MSFT: scenario base Accumulate Carefully, score 76.8, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 1.9%.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 754.68 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 543.45 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 705.82 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 479.45 o peggioramento trend; rischio attuale: Medium-high risk.</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -4316,127 +4294,149 @@
         </is>
       </c>
       <c r="S18" t="n">
-        <v>705.8200000000001</v>
+        <v>479.4474</v>
       </c>
       <c r="T18" t="n">
-        <v>754.6799999999999</v>
-      </c>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
-        </is>
-      </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
+        <v>543.45</v>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr">
         <is>
-          <t>Monitorare ingresso graduale</t>
+          <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y18" t="n">
-        <v>5.49</v>
+        <v>12.51</v>
       </c>
       <c r="Z18" t="n">
-        <v>18.16</v>
+        <v>-2.94</v>
       </c>
       <c r="AA18" t="n">
-        <v>14.13</v>
+        <v>26.13</v>
       </c>
       <c r="AB18" t="n">
-        <v>-23.32</v>
-      </c>
-      <c r="AC18" t="inlineStr"/>
-      <c r="AD18" t="inlineStr"/>
+        <v>-34.5</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>29.07</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>22.02</v>
+      </c>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>Da monitorare: non è un segnale automatico di acquisto.</t>
-        </is>
-      </c>
-      <c r="AF18" t="inlineStr">
-        <is>
-          <t>USA large cap</t>
-        </is>
-      </c>
+          <t>Da monitorare con scenario positivo, base e negativo.</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr"/>
       <c r="AG18" t="n">
-        <v>748.46</v>
-      </c>
-      <c r="AH18" t="n">
-        <v>75.40000000000001</v>
-      </c>
-      <c r="AI18" t="n">
-        <v>69.09999999999999</v>
-      </c>
-      <c r="AJ18" t="n">
-        <v>64.40000000000001</v>
-      </c>
-      <c r="AK18" t="n">
-        <v>82.8</v>
-      </c>
+        <v>521.865</v>
+      </c>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
       <c r="AL18" t="n">
-        <v>2.14</v>
+        <v>1.75</v>
       </c>
       <c r="AM18" t="n">
-        <v>11.47</v>
+        <v>28.5</v>
       </c>
       <c r="AN18" t="n">
-        <v>22.17</v>
+        <v>16.63</v>
       </c>
       <c r="AO18" t="n">
-        <v>1.57</v>
+        <v>0.64</v>
       </c>
       <c r="AP18" t="n">
-        <v>729.1408</v>
+        <v>511.9299</v>
       </c>
       <c r="AQ18" t="n">
-        <v>681.5794</v>
+        <v>436.4854</v>
       </c>
       <c r="AR18" t="inlineStr"/>
       <c r="AS18" t="n">
         <v>85</v>
       </c>
       <c r="AT18" t="n">
-        <v>69.09999999999999</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="AU18" t="n">
-        <v>64.40000000000001</v>
+        <v>41</v>
       </c>
       <c r="AV18" t="n">
         <v>82.8</v>
       </c>
       <c r="AW18" t="n">
-        <v>760</v>
+        <v>753</v>
       </c>
       <c r="AX18" t="n">
-        <v>738.04</v>
+        <v>517.53</v>
       </c>
       <c r="AY18" t="n">
-        <v>754.6799999999999</v>
+        <v>543.45</v>
       </c>
       <c r="AZ18" t="n">
-        <v>2.65</v>
+        <v>1.92</v>
       </c>
       <c r="BA18" t="n">
-        <v>9.81</v>
-      </c>
-      <c r="BB18" t="inlineStr"/>
-      <c r="BC18" t="inlineStr"/>
-      <c r="BD18" t="inlineStr"/>
-      <c r="BE18" t="inlineStr"/>
-      <c r="BF18" t="inlineStr"/>
-      <c r="BG18" t="inlineStr"/>
-      <c r="BH18" t="inlineStr"/>
-      <c r="BI18" t="inlineStr"/>
-      <c r="BJ18" t="inlineStr"/>
-      <c r="BK18" t="inlineStr"/>
-      <c r="BL18" t="inlineStr"/>
-      <c r="BM18" t="inlineStr"/>
-      <c r="BN18" t="inlineStr"/>
+        <v>19.53</v>
+      </c>
+      <c r="BB18" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="BC18" t="inlineStr">
+        <is>
+          <t>Software - Infrastructure</t>
+        </is>
+      </c>
+      <c r="BD18" t="n">
+        <v>3874204155904</v>
+      </c>
+      <c r="BE18" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="BF18" t="n">
+        <v>34.04</v>
+      </c>
+      <c r="BG18" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="BH18" t="n">
+        <v>29.12</v>
+      </c>
+      <c r="BI18" t="n">
+        <v>74</v>
+      </c>
+      <c r="BJ18" t="n">
+        <v>100</v>
+      </c>
+      <c r="BK18" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="BL18" t="n">
+        <v>63</v>
+      </c>
+      <c r="BM18" t="n">
+        <v>41</v>
+      </c>
+      <c r="BN18" t="n">
+        <v>82.8</v>
+      </c>
       <c r="BO18" t="inlineStr"/>
-      <c r="BP18" t="inlineStr"/>
+      <c r="BP18" t="inlineStr">
+        <is>
+          <t>USA / Technology</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4456,10 +4456,10 @@
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
-        <v>72.90000000000001</v>
+        <v>72.7</v>
       </c>
       <c r="F19" t="n">
-        <v>72.90000000000001</v>
+        <v>72.7</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -4473,7 +4473,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>score 72.9; priority 72.9; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 72.7; priority 72.7; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -4493,7 +4493,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>EXSA.DE: scenario base Accumulate Carefully, score 72.9, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.4%.</t>
+          <t>EXSA.DE: scenario base Accumulate Carefully, score 72.7, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.3%.</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -4544,13 +4544,13 @@
         </is>
       </c>
       <c r="Y19" t="n">
-        <v>-0.03</v>
+        <v>-0.19</v>
       </c>
       <c r="Z19" t="n">
-        <v>16.01</v>
+        <v>15.83</v>
       </c>
       <c r="AA19" t="n">
-        <v>12.7</v>
+        <v>12.69</v>
       </c>
       <c r="AB19" t="n">
         <v>-16.33</v>
@@ -4568,13 +4568,13 @@
         </is>
       </c>
       <c r="AG19" t="n">
-        <v>64.42</v>
+        <v>64.31999999999999</v>
       </c>
       <c r="AH19" t="n">
-        <v>76.09999999999999</v>
+        <v>76</v>
       </c>
       <c r="AI19" t="n">
-        <v>57.3</v>
+        <v>56.9</v>
       </c>
       <c r="AJ19" t="n">
         <v>71.7</v>
@@ -4583,29 +4583,29 @@
         <v>82.8</v>
       </c>
       <c r="AL19" t="n">
-        <v>2.47</v>
+        <v>2.31</v>
       </c>
       <c r="AM19" t="n">
-        <v>5.51</v>
+        <v>5.35</v>
       </c>
       <c r="AN19" t="n">
-        <v>17.76</v>
+        <v>17.7</v>
       </c>
       <c r="AO19" t="n">
-        <v>1.4</v>
+        <v>1.39</v>
       </c>
       <c r="AP19" t="n">
-        <v>63.5128</v>
+        <v>63.5108</v>
       </c>
       <c r="AQ19" t="n">
-        <v>61.6335</v>
+        <v>61.633</v>
       </c>
       <c r="AR19" t="inlineStr"/>
       <c r="AS19" t="n">
         <v>85</v>
       </c>
       <c r="AT19" t="n">
-        <v>57.3</v>
+        <v>56.9</v>
       </c>
       <c r="AU19" t="n">
         <v>71.7</v>
@@ -4620,13 +4620,13 @@
         <v>61.93</v>
       </c>
       <c r="AY19" t="n">
-        <v>64.42</v>
+        <v>64.31999999999999</v>
       </c>
       <c r="AZ19" t="n">
-        <v>1.43</v>
+        <v>1.27</v>
       </c>
       <c r="BA19" t="n">
-        <v>4.52</v>
+        <v>4.36</v>
       </c>
       <c r="BB19" t="inlineStr"/>
       <c r="BC19" t="inlineStr"/>
@@ -4666,7 +4666,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>72.8</v>
+        <v>72.7</v>
       </c>
       <c r="F20" t="n">
         <v>72.5</v>
@@ -4678,12 +4678,12 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 349.69. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 348.99. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout.</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>score 72.8; priority 72.5; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 72.7; priority 72.5; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -4703,12 +4703,12 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>AAPL: scenario base Accumulate Carefully, score 72.8, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 5.2%.</t>
+          <t>AAPL: scenario base Accumulate Carefully, score 72.7, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 5.0%.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 349.69 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 348.99 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -4735,7 +4735,7 @@
         <v>302.25</v>
       </c>
       <c r="T20" t="n">
-        <v>349.69</v>
+        <v>348.99</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
@@ -4750,10 +4750,10 @@
         </is>
       </c>
       <c r="Y20" t="n">
-        <v>13.3</v>
+        <v>13.09</v>
       </c>
       <c r="Z20" t="n">
-        <v>30.48</v>
+        <v>30.23</v>
       </c>
       <c r="AA20" t="n">
         <v>26.79</v>
@@ -4762,10 +4762,10 @@
         <v>-33.36</v>
       </c>
       <c r="AC20" t="n">
-        <v>40.1</v>
+        <v>40.03</v>
       </c>
       <c r="AD20" t="n">
-        <v>36.57</v>
+        <v>36.5</v>
       </c>
       <c r="AE20" t="inlineStr">
         <is>
@@ -4774,42 +4774,42 @@
       </c>
       <c r="AF20" t="inlineStr"/>
       <c r="AG20" t="n">
-        <v>349.7</v>
+        <v>349.03</v>
       </c>
       <c r="AH20" t="inlineStr"/>
       <c r="AI20" t="inlineStr"/>
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
       <c r="AL20" t="n">
-        <v>5.01</v>
+        <v>4.81</v>
       </c>
       <c r="AM20" t="n">
-        <v>29.1</v>
+        <v>28.86</v>
       </c>
       <c r="AN20" t="n">
-        <v>27.8</v>
+        <v>27.72</v>
       </c>
       <c r="AO20" t="n">
-        <v>1.04</v>
+        <v>1.03</v>
       </c>
       <c r="AP20" t="n">
-        <v>332.39</v>
+        <v>332.3766</v>
       </c>
       <c r="AQ20" t="n">
-        <v>295.8463</v>
+        <v>295.8429</v>
       </c>
       <c r="AR20" t="inlineStr"/>
       <c r="AS20" t="n">
         <v>85</v>
       </c>
       <c r="AT20" t="n">
-        <v>93.7</v>
+        <v>93.2</v>
       </c>
       <c r="AU20" t="n">
         <v>41.2</v>
       </c>
       <c r="AV20" t="n">
-        <v>77.90000000000001</v>
+        <v>78.7</v>
       </c>
       <c r="AW20" t="n">
         <v>753</v>
@@ -4818,13 +4818,13 @@
         <v>332.89</v>
       </c>
       <c r="AY20" t="n">
-        <v>349.69</v>
+        <v>348.99</v>
       </c>
       <c r="AZ20" t="n">
-        <v>5.2</v>
+        <v>5</v>
       </c>
       <c r="BA20" t="n">
-        <v>18.2</v>
+        <v>17.96</v>
       </c>
       <c r="BB20" t="inlineStr">
         <is>
@@ -4837,7 +4837,7 @@
         </is>
       </c>
       <c r="BD20" t="n">
-        <v>5103803695104</v>
+        <v>5093806571520</v>
       </c>
       <c r="BE20" t="n">
         <v>27.62</v>
@@ -4858,16 +4858,16 @@
         <v>100</v>
       </c>
       <c r="BK20" t="n">
-        <v>93.7</v>
+        <v>93.2</v>
       </c>
       <c r="BL20" t="n">
-        <v>29.4</v>
+        <v>29.6</v>
       </c>
       <c r="BM20" t="n">
         <v>41.2</v>
       </c>
       <c r="BN20" t="n">
-        <v>77.90000000000001</v>
+        <v>78.7</v>
       </c>
       <c r="BO20" t="inlineStr"/>
       <c r="BP20" t="inlineStr">
@@ -4894,10 +4894,10 @@
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>64.5</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="F21" t="n">
-        <v>65.5</v>
+        <v>65.7</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>score 64.5; priority 65.5; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 64.6; priority 65.7; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -4931,7 +4931,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>EIMI.MI: scenario base Hold / Monitor, score 64.5, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -3.5%.</t>
+          <t>EIMI.MI: scenario base Hold / Monitor, score 64.6, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -3.3%.</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -4982,10 +4982,10 @@
         </is>
       </c>
       <c r="Y21" t="n">
-        <v>1.31</v>
+        <v>1.43</v>
       </c>
       <c r="Z21" t="n">
-        <v>17.84</v>
+        <v>17.98</v>
       </c>
       <c r="AA21" t="n">
         <v>17.35</v>
@@ -5006,50 +5006,50 @@
         </is>
       </c>
       <c r="AG21" t="n">
-        <v>46.05</v>
+        <v>46.105</v>
       </c>
       <c r="AH21" t="n">
-        <v>67.90000000000001</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="AI21" t="n">
-        <v>55.3</v>
+        <v>55.6</v>
       </c>
       <c r="AJ21" t="n">
         <v>63.8</v>
       </c>
       <c r="AK21" t="n">
-        <v>74.59999999999999</v>
+        <v>74.7</v>
       </c>
       <c r="AL21" t="n">
-        <v>-4.62</v>
+        <v>-4.5</v>
       </c>
       <c r="AM21" t="n">
-        <v>-1.59</v>
+        <v>-1.47</v>
       </c>
       <c r="AN21" t="n">
-        <v>19.69</v>
+        <v>19.74</v>
       </c>
       <c r="AO21" t="n">
-        <v>1.13</v>
+        <v>1.14</v>
       </c>
       <c r="AP21" t="n">
-        <v>47.6982</v>
+        <v>47.6993</v>
       </c>
       <c r="AQ21" t="n">
-        <v>45.3705</v>
+        <v>45.3708</v>
       </c>
       <c r="AR21" t="inlineStr"/>
       <c r="AS21" t="n">
         <v>65</v>
       </c>
       <c r="AT21" t="n">
-        <v>55.3</v>
+        <v>55.6</v>
       </c>
       <c r="AU21" t="n">
         <v>63.8</v>
       </c>
       <c r="AV21" t="n">
-        <v>74.59999999999999</v>
+        <v>74.7</v>
       </c>
       <c r="AW21" t="n">
         <v>758</v>
@@ -5061,10 +5061,10 @@
         <v>50.16</v>
       </c>
       <c r="AZ21" t="n">
-        <v>-3.46</v>
+        <v>-3.34</v>
       </c>
       <c r="BA21" t="n">
-        <v>1.5</v>
+        <v>1.62</v>
       </c>
       <c r="BB21" t="inlineStr"/>
       <c r="BC21" t="inlineStr"/>
@@ -5103,7 +5103,7 @@
         <v>55.7</v>
       </c>
       <c r="F22" t="n">
-        <v>58.8</v>
+        <v>58.9</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -5117,7 +5117,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>score 55.7; priority 58.8; trend: Weak; entry zone: Wait for trend repair; risk flag: Normal risk</t>
+          <t>score 55.7; priority 58.9; trend: Weak; entry zone: Wait for trend repair; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -5137,7 +5137,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>SGLD.MI: scenario base Hold / Monitor, score 55.7, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -3.7%.</t>
+          <t>SGLD.MI: scenario base Hold / Monitor, score 55.7, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -3.6%.</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -5188,10 +5188,10 @@
         </is>
       </c>
       <c r="Y22" t="n">
-        <v>2.97</v>
+        <v>3.07</v>
       </c>
       <c r="Z22" t="n">
-        <v>5.24</v>
+        <v>5.33</v>
       </c>
       <c r="AA22" t="n">
         <v>19.04</v>
@@ -5212,50 +5212,50 @@
         </is>
       </c>
       <c r="AG22" t="n">
-        <v>347.31</v>
+        <v>347.62</v>
       </c>
       <c r="AH22" t="n">
         <v>62.9</v>
       </c>
       <c r="AI22" t="n">
-        <v>49.7</v>
+        <v>49.9</v>
       </c>
       <c r="AJ22" t="n">
         <v>59</v>
       </c>
       <c r="AK22" t="n">
-        <v>69.8</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="AL22" t="n">
-        <v>-1.41</v>
+        <v>-1.32</v>
       </c>
       <c r="AM22" t="n">
-        <v>-9.59</v>
+        <v>-9.51</v>
       </c>
       <c r="AN22" t="n">
-        <v>23.98</v>
+        <v>24.02</v>
       </c>
       <c r="AO22" t="n">
         <v>1.26</v>
       </c>
       <c r="AP22" t="n">
-        <v>360.5222</v>
+        <v>360.5284</v>
       </c>
       <c r="AQ22" t="n">
-        <v>373.9014</v>
+        <v>373.9029</v>
       </c>
       <c r="AR22" t="inlineStr"/>
       <c r="AS22" t="n">
         <v>35</v>
       </c>
       <c r="AT22" t="n">
-        <v>49.7</v>
+        <v>49.9</v>
       </c>
       <c r="AU22" t="n">
         <v>59</v>
       </c>
       <c r="AV22" t="n">
-        <v>69.8</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="AW22" t="n">
         <v>758</v>
@@ -5267,10 +5267,10 @@
         <v>359.96</v>
       </c>
       <c r="AZ22" t="n">
-        <v>-3.66</v>
+        <v>-3.58</v>
       </c>
       <c r="BA22" t="n">
-        <v>-7.11</v>
+        <v>-7.03</v>
       </c>
       <c r="BB22" t="inlineStr"/>
       <c r="BC22" t="inlineStr"/>

</xml_diff>